<commit_message>
Update New Data.xlsx with latest data revisions
</commit_message>
<xml_diff>
--- a/Data/New Data.xlsx
+++ b/Data/New Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wrca-my.sharepoint.com/personal/huj26_mywrca_ca/Documents/12/Chemistry HL/Chemistry IA/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1996" documentId="8_{ED69E5BD-9A97-5849-9651-1A764BC4410F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF524338-A3A2-E141-AE0C-5CA4233B410D}"/>
+  <xr:revisionPtr revIDLastSave="1998" documentId="8_{ED69E5BD-9A97-5849-9651-1A764BC4410F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB425DEA-C1A6-E945-AD69-455E2FDEC225}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{3196E468-6A35-EA40-9409-42F714E37880}"/>
   </bookViews>
@@ -7495,8 +7495,8 @@
         <v>0.3</v>
       </c>
       <c r="L3" s="170">
-        <f>(250-J3)*0.00001</f>
-        <v>2.2500000000000003E-3</v>
+        <f>(250-J3)*0.000001</f>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M3" s="90"/>
       <c r="O3" s="41" t="s">
@@ -7538,8 +7538,8 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="L4" s="170">
-        <f t="shared" ref="L4:L42" si="1">250-J4</f>
-        <v>225</v>
+        <f t="shared" ref="L4:L42" si="1">(250-J4)*0.000001</f>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M4" s="91"/>
       <c r="O4" s="12" t="s">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="L5" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M5" s="91"/>
       <c r="O5" s="12" t="s">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="L6" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M6" s="91"/>
       <c r="O6" s="12" t="s">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="L7" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M7" s="92" t="s">
         <v>45</v>
@@ -7720,7 +7720,7 @@
       </c>
       <c r="L8" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M8" s="91"/>
       <c r="O8" s="12" t="s">
@@ -7763,7 +7763,7 @@
       </c>
       <c r="L9" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M9" s="91"/>
       <c r="O9" s="13" t="s">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="L10" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M10" s="91"/>
     </row>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="L11" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M11" s="91"/>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="L12" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M12" s="91"/>
     </row>
@@ -7914,7 +7914,7 @@
       </c>
       <c r="L13" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M13" s="91"/>
     </row>
@@ -7947,7 +7947,7 @@
       </c>
       <c r="L14" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M14" s="91"/>
     </row>
@@ -7980,7 +7980,7 @@
       </c>
       <c r="L15" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M15" s="91"/>
     </row>
@@ -8013,7 +8013,7 @@
       </c>
       <c r="L16" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M16" s="91"/>
     </row>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="L17" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M17" s="91"/>
     </row>
@@ -8088,7 +8088,7 @@
       </c>
       <c r="L18" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M18" s="91"/>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="L19" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M19" s="91"/>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="L20" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M20" s="91"/>
     </row>
@@ -8187,7 +8187,7 @@
       </c>
       <c r="L21" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M21" s="91"/>
     </row>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="L22" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M22" s="91"/>
     </row>
@@ -8262,7 +8262,7 @@
       </c>
       <c r="L23" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M23" s="91"/>
     </row>
@@ -8295,7 +8295,7 @@
       </c>
       <c r="L24" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M24" s="91"/>
     </row>
@@ -8328,7 +8328,7 @@
       </c>
       <c r="L25" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M25" s="91"/>
     </row>
@@ -8361,7 +8361,7 @@
       </c>
       <c r="L26" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M26" s="91"/>
     </row>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="L27" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M27" s="91"/>
     </row>
@@ -8436,7 +8436,7 @@
       </c>
       <c r="L28" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M28" s="91"/>
     </row>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="L29" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M29" s="91"/>
     </row>
@@ -8502,7 +8502,7 @@
       </c>
       <c r="L30" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M30" s="91"/>
     </row>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="L31" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M31" s="91"/>
     </row>
@@ -8568,7 +8568,7 @@
       </c>
       <c r="L32" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M32" s="91"/>
     </row>
@@ -8610,7 +8610,7 @@
       </c>
       <c r="L33" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M33" s="91"/>
     </row>
@@ -8643,7 +8643,7 @@
       </c>
       <c r="L34" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M34" s="91"/>
     </row>
@@ -8676,7 +8676,7 @@
       </c>
       <c r="L35" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M35" s="91"/>
     </row>
@@ -8709,7 +8709,7 @@
       </c>
       <c r="L36" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M36" s="91"/>
     </row>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="L37" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M37" s="91"/>
     </row>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="L38" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M38" s="91"/>
     </row>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="L39" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M39" s="91"/>
     </row>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="L40" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M40" s="91"/>
     </row>
@@ -8883,7 +8883,7 @@
       </c>
       <c r="L41" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M41" s="93"/>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="L42" s="170">
         <f t="shared" si="1"/>
-        <v>225</v>
+        <v>2.2499999999999999E-4</v>
       </c>
       <c r="M42" s="94"/>
     </row>

</xml_diff>

<commit_message>
march 1 backup before moving to data analysis
</commit_message>
<xml_diff>
--- a/Data/New Data.xlsx
+++ b/Data/New Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wrca-my.sharepoint.com/personal/huj26_mywrca_ca/Documents/12/Chemistry HL/Chemistry IA/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3100" documentId="8_{ED69E5BD-9A97-5849-9651-1A764BC4410F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB356A82-BADE-2E46-8269-6AD6780D820F}"/>
+  <xr:revisionPtr revIDLastSave="3202" documentId="8_{ED69E5BD-9A97-5849-9651-1A764BC4410F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6277460E-AFA0-2145-9A5F-ADD766D5F4EF}"/>
   <bookViews>
     <workbookView xWindow="-36000" yWindow="16120" windowWidth="36000" windowHeight="22500" activeTab="1" xr2:uid="{3196E468-6A35-EA40-9409-42F714E37880}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="72">
   <si>
     <t>Target (°C)</t>
   </si>
@@ -278,6 +278,24 @@
   </si>
   <si>
     <t>Δln(rate)</t>
+  </si>
+  <si>
+    <t>Random Uncertainty (mol/s)</t>
+  </si>
+  <si>
+    <t>Uncertainty in Avg. Rate (mol/s)</t>
+  </si>
+  <si>
+    <t>Oxygen production rate (mol/s)</t>
+  </si>
+  <si>
+    <t>Δm (Pa/s)</t>
+  </si>
+  <si>
+    <t>Average Δm (Pa/s)</t>
+  </si>
+  <si>
+    <t>Average Slope (Pa/s)</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="276">
+  <cellXfs count="286">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1994,6 +2012,15 @@
     <xf numFmtId="2" fontId="2" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="169" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2109,6 +2136,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="2" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="6" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="2" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="6" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2245,8 +2293,8 @@
             <c:trendlineLbl>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="7.2650161741900417E-3"/>
-                  <c:y val="9.9746850931699785E-2"/>
+                  <c:x val="2.8886530115866657E-2"/>
+                  <c:y val="-5.9893677072666962E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:tx>
@@ -2323,66 +2371,66 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>'Processed Data'!$Q$3:$Q$42</c:f>
+                <c:f>'Processed Data'!$S$3:$S$42</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="40"/>
                   <c:pt idx="0">
-                    <c:v>3.6872643964940771E-7</c:v>
+                    <c:v>1.7596985360013531E-7</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>9.882695021731592E-7</c:v>
+                    <c:v>4.4370293644599947E-7</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>6.3719058620950689E-7</c:v>
+                    <c:v>2.8822893176888274E-7</c:v>
                   </c:pt>
                   <c:pt idx="15">
-                    <c:v>2.6673929684094582E-6</c:v>
+                    <c:v>1.1955215397196222E-6</c:v>
                   </c:pt>
                   <c:pt idx="20">
-                    <c:v>2.0709701812871915E-6</c:v>
+                    <c:v>9.2923209561911543E-7</c:v>
                   </c:pt>
                   <c:pt idx="25">
-                    <c:v>2.7014714463734948E-6</c:v>
+                    <c:v>1.2117876573322692E-6</c:v>
                   </c:pt>
                   <c:pt idx="30">
-                    <c:v>6.0580013453342243E-6</c:v>
+                    <c:v>2.711288692750651E-6</c:v>
                   </c:pt>
                   <c:pt idx="35">
-                    <c:v>8.5359345829324183E-6</c:v>
+                    <c:v>3.820488923827413E-6</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>'Processed Data'!$Q$3:$Q$42</c:f>
+                <c:f>'Processed Data'!$S$3:$S$42</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="40"/>
                   <c:pt idx="0">
-                    <c:v>3.6872643964940771E-7</c:v>
+                    <c:v>1.7596985360013531E-7</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>9.882695021731592E-7</c:v>
+                    <c:v>4.4370293644599947E-7</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>6.3719058620950689E-7</c:v>
+                    <c:v>2.8822893176888274E-7</c:v>
                   </c:pt>
                   <c:pt idx="15">
-                    <c:v>2.6673929684094582E-6</c:v>
+                    <c:v>1.1955215397196222E-6</c:v>
                   </c:pt>
                   <c:pt idx="20">
-                    <c:v>2.0709701812871915E-6</c:v>
+                    <c:v>9.2923209561911543E-7</c:v>
                   </c:pt>
                   <c:pt idx="25">
-                    <c:v>2.7014714463734948E-6</c:v>
+                    <c:v>1.2117876573322692E-6</c:v>
                   </c:pt>
                   <c:pt idx="30">
-                    <c:v>6.0580013453342243E-6</c:v>
+                    <c:v>2.711288692750651E-6</c:v>
                   </c:pt>
                   <c:pt idx="35">
-                    <c:v>8.5359345829324183E-6</c:v>
+                    <c:v>3.820488923827413E-6</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -2532,7 +2580,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Processed Data'!$P$3:$P$42</c:f>
+              <c:f>'Processed Data'!$T$3:$T$42</c:f>
               <c:numCache>
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="40"/>
@@ -7685,13 +7733,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
+      <xdr:col>22</xdr:col>
       <xdr:colOff>8912</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>155964</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>534736</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>101600</xdr:rowOff>
@@ -9771,7 +9819,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBDC91D6-17D9-9B43-8128-D1F89723CF23}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:Z42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" style="1" customWidth="1"/>
@@ -9786,20 +9834,24 @@
     <col min="11" max="11" width="14.6640625" style="1" customWidth="1"/>
     <col min="12" max="12" width="8" style="1" customWidth="1"/>
     <col min="13" max="13" width="19.33203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="31.1640625" style="156" customWidth="1"/>
-    <col min="15" max="15" width="26.33203125" style="166" customWidth="1"/>
-    <col min="16" max="16" width="30" style="166" customWidth="1"/>
-    <col min="17" max="17" width="25.5" style="201" customWidth="1"/>
-    <col min="18" max="18" width="10.83203125" style="1"/>
-    <col min="19" max="19" width="28" style="1" customWidth="1"/>
-    <col min="20" max="20" width="9.6640625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="11.33203125" style="1" customWidth="1"/>
-    <col min="22" max="23" width="10.83203125" style="1"/>
-    <col min="24" max="24" width="13.5" style="1" customWidth="1"/>
-    <col min="25" max="16384" width="10.83203125" style="1"/>
+    <col min="14" max="14" width="11.33203125" style="161" customWidth="1"/>
+    <col min="15" max="15" width="31.1640625" style="156" customWidth="1"/>
+    <col min="16" max="16" width="26.33203125" style="166" customWidth="1"/>
+    <col min="17" max="17" width="20.5" style="166" customWidth="1"/>
+    <col min="18" max="18" width="21.83203125" style="166" customWidth="1"/>
+    <col min="19" max="19" width="30.33203125" style="166" customWidth="1"/>
+    <col min="20" max="20" width="25.6640625" style="166" customWidth="1"/>
+    <col min="21" max="21" width="25.5" style="201" customWidth="1"/>
+    <col min="22" max="22" width="10.83203125" style="1"/>
+    <col min="23" max="23" width="28" style="1" customWidth="1"/>
+    <col min="24" max="24" width="9.6640625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="11.33203125" style="1" customWidth="1"/>
+    <col min="26" max="27" width="10.83203125" style="1"/>
+    <col min="28" max="28" width="13.5" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="125" t="s">
         <v>14</v>
       </c>
@@ -9818,13 +9870,17 @@
       <c r="N1" s="138"/>
       <c r="O1" s="138"/>
       <c r="P1" s="138"/>
-      <c r="Q1" s="127"/>
-      <c r="S1" s="175"/>
-      <c r="T1" s="175"/>
-      <c r="U1" s="175"/>
-      <c r="V1" s="175"/>
+      <c r="Q1" s="138"/>
+      <c r="R1" s="138"/>
+      <c r="S1" s="138"/>
+      <c r="T1" s="138"/>
+      <c r="U1" s="127"/>
+      <c r="W1" s="175"/>
+      <c r="X1" s="175"/>
+      <c r="Y1" s="175"/>
+      <c r="Z1" s="175"/>
     </row>
-    <row r="2" spans="1:22" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -9864,24 +9920,36 @@
       <c r="M2" s="106" t="s">
         <v>53</v>
       </c>
-      <c r="N2" s="164" t="s">
-        <v>52</v>
-      </c>
-      <c r="O2" s="206" t="s">
+      <c r="N2" s="282" t="s">
+        <v>69</v>
+      </c>
+      <c r="O2" s="164" t="s">
+        <v>68</v>
+      </c>
+      <c r="P2" s="206" t="s">
         <v>55</v>
       </c>
-      <c r="P2" s="165" t="s">
-        <v>56</v>
-      </c>
-      <c r="Q2" s="164" t="s">
+      <c r="Q2" s="206" t="s">
+        <v>71</v>
+      </c>
+      <c r="R2" s="206" t="s">
+        <v>70</v>
+      </c>
+      <c r="S2" s="206" t="s">
+        <v>67</v>
+      </c>
+      <c r="T2" s="165" t="s">
+        <v>66</v>
+      </c>
+      <c r="U2" s="164" t="s">
         <v>57</v>
       </c>
-      <c r="S2" s="99"/>
-      <c r="T2" s="99"/>
-      <c r="U2" s="99"/>
-      <c r="V2" s="99"/>
+      <c r="W2" s="99"/>
+      <c r="X2" s="99"/>
+      <c r="Y2" s="99"/>
+      <c r="Z2" s="99"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" s="137">
         <v>1</v>
       </c>
@@ -9898,7 +9966,7 @@
       <c r="E3" s="172">
         <v>14.75</v>
       </c>
-      <c r="F3" s="273">
+      <c r="F3" s="276">
         <f>E3+273.15</f>
         <v>287.89999999999998</v>
       </c>
@@ -9925,24 +9993,39 @@
         <f>L3/(K3-J3)*1000</f>
         <v>14.864864864864863</v>
       </c>
-      <c r="N3" s="191">
+      <c r="N3" s="237">
+        <v>0.45700000000000002</v>
+      </c>
+      <c r="O3" s="191">
         <f>(H3*M3)/(8.31*D3)</f>
         <v>1.3967665818668511E-6</v>
       </c>
-      <c r="O3" s="195">
+      <c r="P3" s="195">
+        <f>AVERAGE(O3:O7)</f>
+        <v>1.8865631315524851E-6</v>
+      </c>
+      <c r="Q3" s="279">
+        <f>AVERAGE(M3:M7)</f>
+        <v>20.077446277446278</v>
+      </c>
+      <c r="R3" s="279">
         <f>AVERAGE(N3:N7)</f>
-        <v>1.8865631315524851E-6</v>
-      </c>
-      <c r="P3" s="202">
-        <f>Q3/SQRT(5)</f>
+        <v>0.65279999999999994</v>
+      </c>
+      <c r="S3" s="279">
+        <f>SQRT(T3^2+((SQRT((0.5/D3)^2+(R3/Q3)^2+(0.06/225)^2))*P3)^2)</f>
+        <v>1.7596985360013531E-7</v>
+      </c>
+      <c r="T3" s="202">
+        <f>U3/SQRT(5)</f>
         <v>1.6489947683150986E-7</v>
       </c>
-      <c r="Q3" s="198">
-        <f>_xlfn.STDEV.S(N3:N7)</f>
+      <c r="U3" s="198">
+        <f>_xlfn.STDEV.S(O3:O7)</f>
         <v>3.6872643964940771E-7</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" s="116"/>
       <c r="B4" s="168">
         <v>2</v>
@@ -9984,15 +10067,21 @@
         <f t="shared" ref="M4:M42" si="3">L4/(K4-J4)*1000</f>
         <v>20.634920634920636</v>
       </c>
-      <c r="N4" s="183">
+      <c r="N4" s="238">
+        <v>1.5109999999999999</v>
+      </c>
+      <c r="O4" s="183">
         <f>(H4*M4)/(8.31*D4)</f>
         <v>1.9389458178295975E-6</v>
       </c>
-      <c r="O4" s="196"/>
-      <c r="P4" s="203"/>
-      <c r="Q4" s="199"/>
+      <c r="P4" s="196"/>
+      <c r="Q4" s="280"/>
+      <c r="R4" s="280"/>
+      <c r="S4" s="280"/>
+      <c r="T4" s="203"/>
+      <c r="U4" s="199"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="116"/>
       <c r="B5" s="168">
         <v>3</v>
@@ -10034,15 +10123,21 @@
         <f t="shared" si="3"/>
         <v>25.666666666666668</v>
       </c>
-      <c r="N5" s="183">
-        <f t="shared" ref="N5:N42" si="4">(H5*M5)/(8.31*D5)</f>
+      <c r="N5" s="238">
+        <v>0.50800000000000001</v>
+      </c>
+      <c r="O5" s="183">
+        <f t="shared" ref="O5:O42" si="4">(H5*M5)/(8.31*D5)</f>
         <v>2.4117502980234296E-6</v>
       </c>
-      <c r="O5" s="196"/>
-      <c r="P5" s="203"/>
-      <c r="Q5" s="199"/>
+      <c r="P5" s="196"/>
+      <c r="Q5" s="280"/>
+      <c r="R5" s="280"/>
+      <c r="S5" s="280"/>
+      <c r="T5" s="203"/>
+      <c r="U5" s="199"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="116"/>
       <c r="B6" s="168">
         <v>4</v>
@@ -10084,15 +10179,21 @@
         <f t="shared" si="3"/>
         <v>20.714285714285712</v>
       </c>
-      <c r="N6" s="183">
+      <c r="N6" s="238">
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="O6" s="183">
         <f t="shared" si="4"/>
         <v>1.9464033017443261E-6</v>
       </c>
-      <c r="O6" s="196"/>
-      <c r="P6" s="203"/>
-      <c r="Q6" s="199"/>
+      <c r="P6" s="196"/>
+      <c r="Q6" s="280"/>
+      <c r="R6" s="280"/>
+      <c r="S6" s="280"/>
+      <c r="T6" s="203"/>
+      <c r="U6" s="199"/>
     </row>
-    <row r="7" spans="1:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="129"/>
       <c r="B7" s="169">
         <v>5</v>
@@ -10134,15 +10235,21 @@
         <f t="shared" si="3"/>
         <v>18.506493506493506</v>
       </c>
-      <c r="N7" s="194">
+      <c r="N7" s="283">
+        <v>0.38</v>
+      </c>
+      <c r="O7" s="194">
         <f t="shared" si="4"/>
         <v>1.7389496582982224E-6</v>
       </c>
-      <c r="O7" s="197"/>
-      <c r="P7" s="204"/>
-      <c r="Q7" s="200"/>
+      <c r="P7" s="197"/>
+      <c r="Q7" s="281"/>
+      <c r="R7" s="281"/>
+      <c r="S7" s="281"/>
+      <c r="T7" s="204"/>
+      <c r="U7" s="200"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="119">
         <v>2</v>
       </c>
@@ -10159,7 +10266,7 @@
       <c r="E8" s="173">
         <v>19</v>
       </c>
-      <c r="F8" s="273">
+      <c r="F8" s="276">
         <f t="shared" si="1"/>
         <v>292.14999999999998</v>
       </c>
@@ -10186,24 +10293,39 @@
         <f t="shared" si="3"/>
         <v>1.8085106382978722</v>
       </c>
-      <c r="N8" s="189">
+      <c r="N8" s="284">
+        <v>0.372</v>
+      </c>
+      <c r="O8" s="189">
         <f t="shared" si="4"/>
         <v>1.6703699313918148E-7</v>
       </c>
-      <c r="O8" s="196">
-        <f t="shared" ref="O8" si="5">AVERAGE(N8:N12)</f>
+      <c r="P8" s="196">
+        <f t="shared" ref="P8" si="5">AVERAGE(O8:O12)</f>
         <v>1.8850179159692152E-6</v>
       </c>
-      <c r="P8" s="203">
-        <f t="shared" ref="P8" si="6">Q8/SQRT(5)</f>
+      <c r="Q8" s="279">
+        <f t="shared" ref="Q8" si="6">AVERAGE(M8:M12)</f>
+        <v>20.409101542984796</v>
+      </c>
+      <c r="R8" s="279">
+        <f t="shared" ref="R8" si="7">AVERAGE(N8:N12)</f>
+        <v>0.42299999999999993</v>
+      </c>
+      <c r="S8" s="279">
+        <f t="shared" ref="S8" si="8">SQRT(T8^2+((SQRT((0.5/D8)^2+(R8/Q8)^2+(0.06/225)^2))*P8)^2)</f>
+        <v>4.4370293644599947E-7</v>
+      </c>
+      <c r="T8" s="203">
+        <f t="shared" ref="T8" si="9">U8/SQRT(5)</f>
         <v>4.4196755738981199E-7</v>
       </c>
-      <c r="Q8" s="199">
-        <f t="shared" ref="Q8" si="7">_xlfn.STDEV.S(N8:N12)</f>
+      <c r="U8" s="199">
+        <f t="shared" ref="U8" si="10">_xlfn.STDEV.S(O8:O12)</f>
         <v>9.882695021731592E-7</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="116"/>
       <c r="B9" s="168">
         <v>2</v>
@@ -10212,7 +10334,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="53">
-        <f t="shared" ref="D9:D42" si="8">C9+273.15</f>
+        <f t="shared" ref="D9:D42" si="11">C9+273.15</f>
         <v>293.14999999999998</v>
       </c>
       <c r="E9" s="173">
@@ -10245,15 +10367,21 @@
         <f t="shared" si="3"/>
         <v>28.125</v>
       </c>
-      <c r="N9" s="183">
+      <c r="N9" s="238">
+        <v>0.432</v>
+      </c>
+      <c r="O9" s="183">
         <f t="shared" si="4"/>
         <v>2.5976708859512412E-6</v>
       </c>
-      <c r="O9" s="196"/>
-      <c r="P9" s="203"/>
-      <c r="Q9" s="199"/>
+      <c r="P9" s="196"/>
+      <c r="Q9" s="280"/>
+      <c r="R9" s="280"/>
+      <c r="S9" s="280"/>
+      <c r="T9" s="203"/>
+      <c r="U9" s="199"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="116"/>
       <c r="B10" s="168">
         <v>3</v>
@@ -10262,7 +10390,7 @@
         <v>20</v>
       </c>
       <c r="D10" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>293.14999999999998</v>
       </c>
       <c r="E10" s="173">
@@ -10295,15 +10423,21 @@
         <f t="shared" si="3"/>
         <v>24.418604651162791</v>
       </c>
-      <c r="N10" s="183">
+      <c r="N10" s="238">
+        <v>0.39</v>
+      </c>
+      <c r="O10" s="183">
         <f t="shared" si="4"/>
         <v>2.2553421645468143E-6</v>
       </c>
-      <c r="O10" s="196"/>
-      <c r="P10" s="203"/>
-      <c r="Q10" s="199"/>
+      <c r="P10" s="196"/>
+      <c r="Q10" s="280"/>
+      <c r="R10" s="280"/>
+      <c r="S10" s="280"/>
+      <c r="T10" s="203"/>
+      <c r="U10" s="199"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="116"/>
       <c r="B11" s="168">
         <v>4</v>
@@ -10312,7 +10446,7 @@
         <v>20</v>
       </c>
       <c r="D11" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>293.14999999999998</v>
       </c>
       <c r="E11" s="173">
@@ -10345,15 +10479,21 @@
         <f t="shared" si="3"/>
         <v>26.369863013698634</v>
       </c>
-      <c r="N11" s="183">
+      <c r="N11" s="238">
+        <v>0.46</v>
+      </c>
+      <c r="O11" s="183">
         <f t="shared" si="4"/>
         <v>2.4355635703895964E-6</v>
       </c>
-      <c r="O11" s="196"/>
-      <c r="P11" s="203"/>
-      <c r="Q11" s="199"/>
+      <c r="P11" s="196"/>
+      <c r="Q11" s="280"/>
+      <c r="R11" s="280"/>
+      <c r="S11" s="280"/>
+      <c r="T11" s="203"/>
+      <c r="U11" s="199"/>
     </row>
-    <row r="12" spans="1:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="128"/>
       <c r="B12" s="171">
         <v>5</v>
@@ -10362,7 +10502,7 @@
         <v>20</v>
       </c>
       <c r="D12" s="208">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>293.14999999999998</v>
       </c>
       <c r="E12" s="209">
@@ -10395,15 +10535,21 @@
         <f t="shared" si="3"/>
         <v>21.323529411764703</v>
       </c>
-      <c r="N12" s="213">
+      <c r="N12" s="285">
+        <v>0.46100000000000002</v>
+      </c>
+      <c r="O12" s="213">
         <f t="shared" si="4"/>
         <v>1.9694759658192417E-6</v>
       </c>
-      <c r="O12" s="196"/>
-      <c r="P12" s="203"/>
-      <c r="Q12" s="199"/>
+      <c r="P12" s="196"/>
+      <c r="Q12" s="281"/>
+      <c r="R12" s="281"/>
+      <c r="S12" s="281"/>
+      <c r="T12" s="203"/>
+      <c r="U12" s="199"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="137">
         <v>3</v>
       </c>
@@ -10414,13 +10560,13 @@
         <v>25</v>
       </c>
       <c r="D13" s="52">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>298.14999999999998</v>
       </c>
       <c r="E13" s="172">
         <v>25.5</v>
       </c>
-      <c r="F13" s="273">
+      <c r="F13" s="276">
         <f t="shared" si="1"/>
         <v>298.64999999999998</v>
       </c>
@@ -10447,24 +10593,39 @@
         <f t="shared" si="3"/>
         <v>42.715231788079471</v>
       </c>
-      <c r="N13" s="191">
+      <c r="N13" s="237">
+        <v>0.41499999999999998</v>
+      </c>
+      <c r="O13" s="191">
         <f t="shared" si="4"/>
         <v>3.8790863563648034E-6</v>
       </c>
-      <c r="O13" s="195">
-        <f t="shared" ref="O13" si="9">AVERAGE(N13:N17)</f>
+      <c r="P13" s="195">
+        <f t="shared" ref="P13" si="12">AVERAGE(O13:O17)</f>
         <v>3.3903837799776504E-6</v>
       </c>
-      <c r="P13" s="202">
-        <f t="shared" ref="P13" si="10">Q13/SQRT(5)</f>
+      <c r="Q13" s="279">
+        <f t="shared" ref="Q13" si="13">AVERAGE(M13:M17)</f>
+        <v>37.333798659745767</v>
+      </c>
+      <c r="R13" s="279">
+        <f t="shared" ref="R13" si="14">AVERAGE(N13:N17)</f>
+        <v>0.47240000000000004</v>
+      </c>
+      <c r="S13" s="279">
+        <f t="shared" ref="S13" si="15">SQRT(T13^2+((SQRT((0.5/D13)^2+(R13/Q13)^2+(0.06/225)^2))*P13)^2)</f>
+        <v>2.8822893176888274E-7</v>
+      </c>
+      <c r="T13" s="202">
+        <f t="shared" ref="T13" si="16">U13/SQRT(5)</f>
         <v>2.8496029307747946E-7</v>
       </c>
-      <c r="Q13" s="198">
-        <f t="shared" ref="Q13" si="11">_xlfn.STDEV.S(N13:N17)</f>
+      <c r="U13" s="198">
+        <f t="shared" ref="U13" si="17">_xlfn.STDEV.S(O13:O17)</f>
         <v>6.3719058620950689E-7</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A14" s="116"/>
       <c r="B14" s="168">
         <v>2</v>
@@ -10473,7 +10634,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>298.14999999999998</v>
       </c>
       <c r="E14" s="173">
@@ -10506,15 +10667,21 @@
         <f t="shared" si="3"/>
         <v>46.107784431137731</v>
       </c>
-      <c r="N14" s="183">
+      <c r="N14" s="238">
+        <v>0.44500000000000001</v>
+      </c>
+      <c r="O14" s="183">
         <f t="shared" si="4"/>
         <v>4.1871732874208404E-6</v>
       </c>
-      <c r="O14" s="196"/>
-      <c r="P14" s="203"/>
-      <c r="Q14" s="199"/>
+      <c r="P14" s="196"/>
+      <c r="Q14" s="280"/>
+      <c r="R14" s="280"/>
+      <c r="S14" s="280"/>
+      <c r="T14" s="203"/>
+      <c r="U14" s="199"/>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" s="116"/>
       <c r="B15" s="168">
         <v>3</v>
@@ -10523,7 +10690,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>298.14999999999998</v>
       </c>
       <c r="E15" s="173">
@@ -10556,15 +10723,21 @@
         <f t="shared" si="3"/>
         <v>34.883720930232563</v>
       </c>
-      <c r="N15" s="183">
+      <c r="N15" s="238">
+        <v>0.50700000000000001</v>
+      </c>
+      <c r="O15" s="183">
         <f t="shared" si="4"/>
         <v>3.1678855587403213E-6</v>
       </c>
-      <c r="O15" s="196"/>
-      <c r="P15" s="203"/>
-      <c r="Q15" s="199"/>
+      <c r="P15" s="196"/>
+      <c r="Q15" s="280"/>
+      <c r="R15" s="280"/>
+      <c r="S15" s="280"/>
+      <c r="T15" s="203"/>
+      <c r="U15" s="199"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A16" s="116"/>
       <c r="B16" s="168">
         <v>4</v>
@@ -10573,7 +10746,7 @@
         <v>25</v>
       </c>
       <c r="D16" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>298.14999999999998</v>
       </c>
       <c r="E16" s="173">
@@ -10606,15 +10779,21 @@
         <f t="shared" si="3"/>
         <v>28.611111111111111</v>
       </c>
-      <c r="N16" s="183">
+      <c r="N16" s="238">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="O16" s="183">
         <f t="shared" si="4"/>
         <v>2.5982528036409038E-6</v>
       </c>
-      <c r="O16" s="196"/>
-      <c r="P16" s="203"/>
-      <c r="Q16" s="199"/>
+      <c r="P16" s="196"/>
+      <c r="Q16" s="280"/>
+      <c r="R16" s="280"/>
+      <c r="S16" s="280"/>
+      <c r="T16" s="203"/>
+      <c r="U16" s="199"/>
     </row>
-    <row r="17" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="129"/>
       <c r="B17" s="170">
         <v>5</v>
@@ -10623,7 +10802,7 @@
         <v>25</v>
       </c>
       <c r="D17" s="54">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>298.14999999999998</v>
       </c>
       <c r="E17" s="174">
@@ -10656,15 +10835,21 @@
         <f t="shared" si="3"/>
         <v>34.351145038167935</v>
       </c>
-      <c r="N17" s="185">
+      <c r="N17" s="239">
+        <v>0.51600000000000001</v>
+      </c>
+      <c r="O17" s="185">
         <f t="shared" si="4"/>
         <v>3.1195208937213843E-6</v>
       </c>
-      <c r="O17" s="197"/>
-      <c r="P17" s="204"/>
-      <c r="Q17" s="200"/>
+      <c r="P17" s="197"/>
+      <c r="Q17" s="281"/>
+      <c r="R17" s="281"/>
+      <c r="S17" s="281"/>
+      <c r="T17" s="204"/>
+      <c r="U17" s="200"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" s="137">
         <v>4</v>
       </c>
@@ -10675,13 +10860,13 @@
         <v>30</v>
       </c>
       <c r="D18" s="52">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>303.14999999999998</v>
       </c>
       <c r="E18" s="172">
         <v>30.1</v>
       </c>
-      <c r="F18" s="273">
+      <c r="F18" s="276">
         <f t="shared" si="1"/>
         <v>303.25</v>
       </c>
@@ -10708,24 +10893,39 @@
         <f t="shared" si="3"/>
         <v>123.39999999999999</v>
       </c>
-      <c r="N18" s="191">
+      <c r="N18" s="237">
+        <v>1.147</v>
+      </c>
+      <c r="O18" s="191">
         <f t="shared" si="4"/>
         <v>1.1021458798142964E-5</v>
       </c>
-      <c r="O18" s="195">
-        <f t="shared" ref="O18" si="12">AVERAGE(N18:N22)</f>
+      <c r="P18" s="195">
+        <f t="shared" ref="P18" si="18">AVERAGE(O18:O22)</f>
         <v>7.5427965937800808E-6</v>
       </c>
-      <c r="P18" s="202">
-        <f t="shared" ref="P18" si="13">Q18/SQRT(5)</f>
+      <c r="Q18" s="279">
+        <f t="shared" ref="Q18" si="19">AVERAGE(M18:M22)</f>
+        <v>84.451715214803684</v>
+      </c>
+      <c r="R18" s="279">
+        <f t="shared" ref="R18" si="20">AVERAGE(N18:N22)</f>
+        <v>0.87560000000000004</v>
+      </c>
+      <c r="S18" s="279">
+        <f t="shared" ref="S18" si="21">SQRT(T18^2+((SQRT((0.5/D18)^2+(R18/Q18)^2+(0.06/225)^2))*P18)^2)</f>
+        <v>1.1955215397196222E-6</v>
+      </c>
+      <c r="T18" s="202">
+        <f t="shared" ref="T18" si="22">U18/SQRT(5)</f>
         <v>1.1928944000136995E-6</v>
       </c>
-      <c r="Q18" s="198">
-        <f t="shared" ref="Q18" si="14">_xlfn.STDEV.S(N18:N22)</f>
+      <c r="U18" s="198">
+        <f t="shared" ref="U18" si="23">_xlfn.STDEV.S(O18:O22)</f>
         <v>2.6673929684094582E-6</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" s="116"/>
       <c r="B19" s="168">
         <v>2</v>
@@ -10734,7 +10934,7 @@
         <v>30</v>
       </c>
       <c r="D19" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>303.14999999999998</v>
       </c>
       <c r="E19" s="173">
@@ -10767,15 +10967,21 @@
         <f t="shared" si="3"/>
         <v>59.442060085836907</v>
       </c>
-      <c r="N19" s="183">
+      <c r="N19" s="238">
+        <v>0.72599999999999998</v>
+      </c>
+      <c r="O19" s="183">
         <f t="shared" si="4"/>
         <v>5.309061718904294E-6</v>
       </c>
-      <c r="O19" s="196"/>
-      <c r="P19" s="203"/>
-      <c r="Q19" s="199"/>
+      <c r="P19" s="196"/>
+      <c r="Q19" s="280"/>
+      <c r="R19" s="280"/>
+      <c r="S19" s="280"/>
+      <c r="T19" s="203"/>
+      <c r="U19" s="199"/>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" s="116"/>
       <c r="B20" s="168">
         <v>3</v>
@@ -10784,7 +10990,7 @@
         <v>30</v>
       </c>
       <c r="D20" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>303.14999999999998</v>
       </c>
       <c r="E20" s="173">
@@ -10817,15 +11023,21 @@
         <f t="shared" si="3"/>
         <v>108.93536121673004</v>
       </c>
-      <c r="N20" s="183">
+      <c r="N20" s="238">
+        <v>1.0740000000000001</v>
+      </c>
+      <c r="O20" s="183">
         <f t="shared" si="4"/>
         <v>9.7295510154863137E-6</v>
       </c>
-      <c r="O20" s="196"/>
-      <c r="P20" s="203"/>
-      <c r="Q20" s="199"/>
+      <c r="P20" s="196"/>
+      <c r="Q20" s="280"/>
+      <c r="R20" s="280"/>
+      <c r="S20" s="280"/>
+      <c r="T20" s="203"/>
+      <c r="U20" s="199"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" s="116"/>
       <c r="B21" s="168">
         <v>4</v>
@@ -10834,7 +11046,7 @@
         <v>30</v>
       </c>
       <c r="D21" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>303.14999999999998</v>
       </c>
       <c r="E21" s="173">
@@ -10867,15 +11079,21 @@
         <f t="shared" si="3"/>
         <v>71.860465116279073</v>
       </c>
-      <c r="N21" s="183">
+      <c r="N21" s="238">
+        <v>0.70099999999999996</v>
+      </c>
+      <c r="O21" s="183">
         <f t="shared" si="4"/>
         <v>6.4182103362598011E-6</v>
       </c>
-      <c r="O21" s="196"/>
-      <c r="P21" s="203"/>
-      <c r="Q21" s="199"/>
+      <c r="P21" s="196"/>
+      <c r="Q21" s="280"/>
+      <c r="R21" s="280"/>
+      <c r="S21" s="280"/>
+      <c r="T21" s="203"/>
+      <c r="U21" s="199"/>
     </row>
-    <row r="22" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="129"/>
       <c r="B22" s="170">
         <v>5</v>
@@ -10884,7 +11102,7 @@
         <v>30</v>
       </c>
       <c r="D22" s="54">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>303.14999999999998</v>
       </c>
       <c r="E22" s="174">
@@ -10917,15 +11135,21 @@
         <f t="shared" si="3"/>
         <v>58.620689655172406</v>
       </c>
-      <c r="N22" s="185">
+      <c r="N22" s="239">
+        <v>0.73</v>
+      </c>
+      <c r="O22" s="185">
         <f t="shared" si="4"/>
         <v>5.2357011001070352E-6</v>
       </c>
-      <c r="O22" s="197"/>
-      <c r="P22" s="204"/>
-      <c r="Q22" s="200"/>
+      <c r="P22" s="197"/>
+      <c r="Q22" s="281"/>
+      <c r="R22" s="281"/>
+      <c r="S22" s="281"/>
+      <c r="T22" s="204"/>
+      <c r="U22" s="200"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23" s="119">
         <v>5</v>
       </c>
@@ -10936,13 +11160,13 @@
         <v>35</v>
       </c>
       <c r="D23" s="205">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
       <c r="E23" s="173">
         <v>35.5</v>
       </c>
-      <c r="F23" s="273">
+      <c r="F23" s="276">
         <f t="shared" si="1"/>
         <v>308.64999999999998</v>
       </c>
@@ -10969,24 +11193,39 @@
         <f t="shared" si="3"/>
         <v>117.24137931034483</v>
       </c>
-      <c r="N23" s="189">
+      <c r="N23" s="284">
+        <v>0.90200000000000002</v>
+      </c>
+      <c r="O23" s="189">
         <f t="shared" si="4"/>
         <v>1.0301494651938654E-5</v>
       </c>
-      <c r="O23" s="196">
-        <f t="shared" ref="O23" si="15">AVERAGE(N23:N27)</f>
+      <c r="P23" s="196">
+        <f t="shared" ref="P23" si="24">AVERAGE(O23:O27)</f>
         <v>8.5940925905051713E-6</v>
       </c>
-      <c r="P23" s="203">
-        <f t="shared" ref="P23" si="16">Q23/SQRT(5)</f>
+      <c r="Q23" s="279">
+        <f t="shared" ref="Q23" si="25">AVERAGE(M23:M27)</f>
+        <v>97.809425066489965</v>
+      </c>
+      <c r="R23" s="279">
+        <f t="shared" ref="R23" si="26">AVERAGE(N23:N27)</f>
+        <v>0.84320000000000006</v>
+      </c>
+      <c r="S23" s="279">
+        <f t="shared" ref="S23" si="27">SQRT(T23^2+((SQRT((0.5/D23)^2+(R23/Q23)^2+(0.06/225)^2))*P23)^2)</f>
+        <v>9.2923209561911543E-7</v>
+      </c>
+      <c r="T23" s="203">
+        <f t="shared" ref="T23" si="28">U23/SQRT(5)</f>
         <v>9.2616602094664455E-7</v>
       </c>
-      <c r="Q23" s="199">
-        <f t="shared" ref="Q23" si="17">_xlfn.STDEV.S(N23:N27)</f>
+      <c r="U23" s="199">
+        <f t="shared" ref="U23" si="29">_xlfn.STDEV.S(O23:O27)</f>
         <v>2.0709701812871915E-6</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" s="116"/>
       <c r="B24" s="168">
         <v>2</v>
@@ -10995,7 +11234,7 @@
         <v>35</v>
       </c>
       <c r="D24" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
       <c r="E24" s="173">
@@ -11028,15 +11267,21 @@
         <f t="shared" si="3"/>
         <v>89.351851851851848</v>
       </c>
-      <c r="N24" s="183">
+      <c r="N24" s="238">
+        <v>0.78500000000000003</v>
+      </c>
+      <c r="O24" s="183">
         <f t="shared" si="4"/>
         <v>7.8509620869962748E-6</v>
       </c>
-      <c r="O24" s="196"/>
-      <c r="P24" s="203"/>
-      <c r="Q24" s="199"/>
+      <c r="P24" s="196"/>
+      <c r="Q24" s="280"/>
+      <c r="R24" s="280"/>
+      <c r="S24" s="280"/>
+      <c r="T24" s="203"/>
+      <c r="U24" s="199"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25" s="116"/>
       <c r="B25" s="168">
         <v>3</v>
@@ -11045,7 +11290,7 @@
         <v>35</v>
       </c>
       <c r="D25" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
       <c r="E25" s="173">
@@ -11078,15 +11323,21 @@
         <f t="shared" si="3"/>
         <v>100.89686098654708</v>
       </c>
-      <c r="N25" s="183">
+      <c r="N25" s="238">
+        <v>0.77</v>
+      </c>
+      <c r="O25" s="183">
         <f t="shared" si="4"/>
         <v>8.8653722769585487E-6</v>
       </c>
-      <c r="O25" s="196"/>
-      <c r="P25" s="203"/>
-      <c r="Q25" s="199"/>
+      <c r="P25" s="196"/>
+      <c r="Q25" s="280"/>
+      <c r="R25" s="280"/>
+      <c r="S25" s="280"/>
+      <c r="T25" s="203"/>
+      <c r="U25" s="199"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A26" s="116"/>
       <c r="B26" s="168">
         <v>4</v>
@@ -11095,7 +11346,7 @@
         <v>35</v>
       </c>
       <c r="D26" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
       <c r="E26" s="173">
@@ -11128,15 +11379,21 @@
         <f t="shared" si="3"/>
         <v>119.62809917355374</v>
       </c>
-      <c r="N26" s="183">
+      <c r="N26" s="238">
+        <v>1.081</v>
+      </c>
+      <c r="O26" s="183">
         <f t="shared" si="4"/>
         <v>1.0511205438788404E-5</v>
       </c>
-      <c r="O26" s="196"/>
-      <c r="P26" s="203"/>
-      <c r="Q26" s="199"/>
+      <c r="P26" s="196"/>
+      <c r="Q26" s="280"/>
+      <c r="R26" s="280"/>
+      <c r="S26" s="280"/>
+      <c r="T26" s="203"/>
+      <c r="U26" s="199"/>
     </row>
-    <row r="27" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="128"/>
       <c r="B27" s="171">
         <v>5</v>
@@ -11145,7 +11402,7 @@
         <v>35</v>
       </c>
       <c r="D27" s="208">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
       <c r="E27" s="209">
@@ -11178,15 +11435,21 @@
         <f t="shared" si="3"/>
         <v>61.92893401015229</v>
       </c>
-      <c r="N27" s="213">
+      <c r="N27" s="285">
+        <v>0.67800000000000005</v>
+      </c>
+      <c r="O27" s="213">
         <f t="shared" si="4"/>
         <v>5.4414284978439773E-6</v>
       </c>
-      <c r="O27" s="196"/>
-      <c r="P27" s="203"/>
-      <c r="Q27" s="199"/>
+      <c r="P27" s="196"/>
+      <c r="Q27" s="281"/>
+      <c r="R27" s="281"/>
+      <c r="S27" s="281"/>
+      <c r="T27" s="203"/>
+      <c r="U27" s="199"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" s="137">
         <v>6</v>
       </c>
@@ -11197,13 +11460,13 @@
         <v>40</v>
       </c>
       <c r="D28" s="52">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>313.14999999999998</v>
       </c>
       <c r="E28" s="172">
         <v>40.349999999999994</v>
       </c>
-      <c r="F28" s="273">
+      <c r="F28" s="276">
         <f t="shared" si="1"/>
         <v>313.5</v>
       </c>
@@ -11230,24 +11493,39 @@
         <f t="shared" si="3"/>
         <v>113.52459016393443</v>
       </c>
-      <c r="N28" s="191">
+      <c r="N28" s="237">
+        <v>1.0409999999999999</v>
+      </c>
+      <c r="O28" s="191">
         <f t="shared" si="4"/>
         <v>9.8156490238009875E-6</v>
       </c>
-      <c r="O28" s="195">
-        <f t="shared" ref="O28" si="18">AVERAGE(N28:N32)</f>
+      <c r="P28" s="195">
+        <f t="shared" ref="P28" si="30">AVERAGE(O28:O32)</f>
         <v>8.8862471284774915E-6</v>
       </c>
-      <c r="P28" s="202">
-        <f t="shared" ref="P28" si="19">Q28/SQRT(5)</f>
+      <c r="Q28" s="279">
+        <f t="shared" ref="Q28" si="31">AVERAGE(M28:M32)</f>
+        <v>102.775431447242</v>
+      </c>
+      <c r="R28" s="279">
+        <f t="shared" ref="R28" si="32">AVERAGE(N28:N32)</f>
+        <v>1.0745999999999998</v>
+      </c>
+      <c r="S28" s="279">
+        <f t="shared" ref="S28" si="33">SQRT(T28^2+((SQRT((0.5/D28)^2+(R28/Q28)^2+(0.06/225)^2))*P28)^2)</f>
+        <v>1.2117876573322692E-6</v>
+      </c>
+      <c r="T28" s="202">
+        <f t="shared" ref="T28" si="34">U28/SQRT(5)</f>
         <v>1.2081347586731623E-6</v>
       </c>
-      <c r="Q28" s="198">
-        <f t="shared" ref="Q28" si="20">_xlfn.STDEV.S(N28:N32)</f>
+      <c r="U28" s="198">
+        <f t="shared" ref="U28" si="35">_xlfn.STDEV.S(O28:O32)</f>
         <v>2.7014714463734948E-6</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29" s="116"/>
       <c r="B29" s="168">
         <v>2</v>
@@ -11256,7 +11534,7 @@
         <v>40</v>
       </c>
       <c r="D29" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>313.14999999999998</v>
       </c>
       <c r="E29" s="173">
@@ -11289,15 +11567,21 @@
         <f t="shared" si="3"/>
         <v>94.68599033816426</v>
       </c>
-      <c r="N29" s="183">
+      <c r="N29" s="238">
+        <v>0.84499999999999997</v>
+      </c>
+      <c r="O29" s="183">
         <f t="shared" si="4"/>
         <v>8.1868117496687828E-6</v>
       </c>
-      <c r="O29" s="196"/>
-      <c r="P29" s="203"/>
-      <c r="Q29" s="199"/>
+      <c r="P29" s="196"/>
+      <c r="Q29" s="280"/>
+      <c r="R29" s="280"/>
+      <c r="S29" s="280"/>
+      <c r="T29" s="203"/>
+      <c r="U29" s="199"/>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30" s="116"/>
       <c r="B30" s="168">
         <v>3</v>
@@ -11306,7 +11590,7 @@
         <v>40</v>
       </c>
       <c r="D30" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>313.14999999999998</v>
       </c>
       <c r="E30" s="173">
@@ -11339,15 +11623,21 @@
         <f t="shared" si="3"/>
         <v>72.146118721461193</v>
       </c>
-      <c r="N30" s="183">
+      <c r="N30" s="238">
+        <v>0.85599999999999998</v>
+      </c>
+      <c r="O30" s="183">
         <f t="shared" si="4"/>
         <v>6.2379523130339029E-6</v>
       </c>
-      <c r="O30" s="196"/>
-      <c r="P30" s="203"/>
-      <c r="Q30" s="199"/>
+      <c r="P30" s="196"/>
+      <c r="Q30" s="280"/>
+      <c r="R30" s="280"/>
+      <c r="S30" s="280"/>
+      <c r="T30" s="203"/>
+      <c r="U30" s="199"/>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A31" s="116"/>
       <c r="B31" s="168">
         <v>4</v>
@@ -11356,7 +11646,7 @@
         <v>40</v>
       </c>
       <c r="D31" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>313.14999999999998</v>
       </c>
       <c r="E31" s="173">
@@ -11389,15 +11679,21 @@
         <f t="shared" si="3"/>
         <v>151.36186770428017</v>
       </c>
-      <c r="N31" s="183">
+      <c r="N31" s="238">
+        <v>1.728</v>
+      </c>
+      <c r="O31" s="183">
         <f t="shared" si="4"/>
         <v>1.3087164347625258E-5</v>
       </c>
-      <c r="O31" s="196"/>
-      <c r="P31" s="203"/>
-      <c r="Q31" s="199"/>
+      <c r="P31" s="196"/>
+      <c r="Q31" s="280"/>
+      <c r="R31" s="280"/>
+      <c r="S31" s="280"/>
+      <c r="T31" s="203"/>
+      <c r="U31" s="199"/>
     </row>
-    <row r="32" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="129"/>
       <c r="B32" s="170">
         <v>5</v>
@@ -11406,7 +11702,7 @@
         <v>40</v>
       </c>
       <c r="D32" s="54">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>313.14999999999998</v>
       </c>
       <c r="E32" s="174">
@@ -11439,15 +11735,21 @@
         <f t="shared" si="3"/>
         <v>82.158590308370037</v>
       </c>
-      <c r="N32" s="185">
+      <c r="N32" s="239">
+        <v>0.90300000000000002</v>
+      </c>
+      <c r="O32" s="185">
         <f t="shared" si="4"/>
         <v>7.1036582082585224E-6</v>
       </c>
-      <c r="O32" s="197"/>
-      <c r="P32" s="204"/>
-      <c r="Q32" s="200"/>
+      <c r="P32" s="197"/>
+      <c r="Q32" s="281"/>
+      <c r="R32" s="281"/>
+      <c r="S32" s="281"/>
+      <c r="T32" s="204"/>
+      <c r="U32" s="200"/>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33" s="137">
         <v>7</v>
       </c>
@@ -11458,13 +11760,13 @@
         <v>45</v>
       </c>
       <c r="D33" s="52">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>318.14999999999998</v>
       </c>
       <c r="E33" s="172">
         <v>45.25</v>
       </c>
-      <c r="F33" s="273">
+      <c r="F33" s="276">
         <f t="shared" si="1"/>
         <v>318.39999999999998</v>
       </c>
@@ -11491,24 +11793,39 @@
         <f t="shared" si="3"/>
         <v>133.39622641509436</v>
       </c>
-      <c r="N33" s="191">
+      <c r="N33" s="237">
+        <v>1.7330000000000001</v>
+      </c>
+      <c r="O33" s="191">
         <f t="shared" si="4"/>
         <v>1.1352541834116659E-5</v>
       </c>
-      <c r="O33" s="195">
-        <f t="shared" ref="O33" si="21">AVERAGE(N33:N37)</f>
+      <c r="P33" s="195">
+        <f t="shared" ref="P33" si="36">AVERAGE(O33:O37)</f>
         <v>1.2906068842991905E-5</v>
       </c>
-      <c r="P33" s="202">
-        <f t="shared" ref="P33" si="22">Q33/SQRT(5)</f>
+      <c r="Q33" s="279">
+        <f t="shared" ref="Q33" si="37">AVERAGE(M33:M37)</f>
+        <v>151.65069696856148</v>
+      </c>
+      <c r="R33" s="279">
+        <f t="shared" ref="R33" si="38">AVERAGE(N33:N37)</f>
+        <v>1.2204000000000002</v>
+      </c>
+      <c r="S33" s="279">
+        <f t="shared" ref="S33" si="39">SQRT(T33^2+((SQRT((0.5/D33)^2+(R33/Q33)^2+(0.06/225)^2))*P33)^2)</f>
+        <v>2.711288692750651E-6</v>
+      </c>
+      <c r="T33" s="202">
+        <f t="shared" ref="T33" si="40">U33/SQRT(5)</f>
         <v>2.7092205631905007E-6</v>
       </c>
-      <c r="Q33" s="198">
-        <f t="shared" ref="Q33" si="23">_xlfn.STDEV.S(N33:N37)</f>
+      <c r="U33" s="198">
+        <f t="shared" ref="U33" si="41">_xlfn.STDEV.S(O33:O37)</f>
         <v>6.0580013453342243E-6</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A34" s="116"/>
       <c r="B34" s="168">
         <v>2</v>
@@ -11517,7 +11834,7 @@
         <v>45</v>
       </c>
       <c r="D34" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>318.14999999999998</v>
       </c>
       <c r="E34" s="173">
@@ -11550,15 +11867,21 @@
         <f t="shared" si="3"/>
         <v>110.55045871559633</v>
       </c>
-      <c r="N34" s="183">
+      <c r="N34" s="238">
+        <v>0.99</v>
+      </c>
+      <c r="O34" s="183">
         <f t="shared" si="4"/>
         <v>9.4082774384057253E-6</v>
       </c>
-      <c r="O34" s="196"/>
-      <c r="P34" s="203"/>
-      <c r="Q34" s="199"/>
+      <c r="P34" s="196"/>
+      <c r="Q34" s="280"/>
+      <c r="R34" s="280"/>
+      <c r="S34" s="280"/>
+      <c r="T34" s="203"/>
+      <c r="U34" s="199"/>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35" s="116"/>
       <c r="B35" s="168">
         <v>3</v>
@@ -11567,7 +11890,7 @@
         <v>45</v>
       </c>
       <c r="D35" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>318.14999999999998</v>
       </c>
       <c r="E35" s="173">
@@ -11600,15 +11923,21 @@
         <f t="shared" si="3"/>
         <v>209.02527075812276</v>
       </c>
-      <c r="N35" s="183">
+      <c r="N35" s="238">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="O35" s="183">
         <f t="shared" si="4"/>
         <v>1.7788870003601831E-5</v>
       </c>
-      <c r="O35" s="196"/>
-      <c r="P35" s="203"/>
-      <c r="Q35" s="199"/>
+      <c r="P35" s="196"/>
+      <c r="Q35" s="280"/>
+      <c r="R35" s="280"/>
+      <c r="S35" s="280"/>
+      <c r="T35" s="203"/>
+      <c r="U35" s="199"/>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A36" s="116"/>
       <c r="B36" s="168">
         <v>4</v>
@@ -11617,7 +11946,7 @@
         <v>45</v>
       </c>
       <c r="D36" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>318.14999999999998</v>
       </c>
       <c r="E36" s="173">
@@ -11650,15 +11979,21 @@
         <f t="shared" si="3"/>
         <v>239.10505836575874</v>
       </c>
-      <c r="N36" s="183">
+      <c r="N36" s="238">
+        <v>1.6619999999999999</v>
+      </c>
+      <c r="O36" s="183">
         <f t="shared" si="4"/>
         <v>2.0348777853726677E-5</v>
       </c>
-      <c r="O36" s="196"/>
-      <c r="P36" s="203"/>
-      <c r="Q36" s="199"/>
+      <c r="P36" s="196"/>
+      <c r="Q36" s="280"/>
+      <c r="R36" s="280"/>
+      <c r="S36" s="280"/>
+      <c r="T36" s="203"/>
+      <c r="U36" s="199"/>
     </row>
-    <row r="37" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="129"/>
       <c r="B37" s="170">
         <v>5</v>
@@ -11667,7 +12002,7 @@
         <v>45</v>
       </c>
       <c r="D37" s="54">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>318.14999999999998</v>
       </c>
       <c r="E37" s="174">
@@ -11700,15 +12035,21 @@
         <f t="shared" si="3"/>
         <v>66.17647058823529</v>
       </c>
-      <c r="N37" s="185">
+      <c r="N37" s="239">
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="O37" s="185">
         <f t="shared" si="4"/>
         <v>5.6318770851086252E-6</v>
       </c>
-      <c r="O37" s="197"/>
-      <c r="P37" s="204"/>
-      <c r="Q37" s="200"/>
+      <c r="P37" s="197"/>
+      <c r="Q37" s="281"/>
+      <c r="R37" s="281"/>
+      <c r="S37" s="281"/>
+      <c r="T37" s="204"/>
+      <c r="U37" s="200"/>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A38" s="119">
         <v>8</v>
       </c>
@@ -11719,13 +12060,13 @@
         <v>50</v>
       </c>
       <c r="D38" s="205">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>323.14999999999998</v>
       </c>
       <c r="E38" s="173">
         <v>49.3</v>
       </c>
-      <c r="F38" s="273">
+      <c r="F38" s="276">
         <f t="shared" si="1"/>
         <v>322.45</v>
       </c>
@@ -11752,24 +12093,39 @@
         <f t="shared" si="3"/>
         <v>368.34677419354841</v>
       </c>
-      <c r="N38" s="189">
+      <c r="N38" s="284">
+        <v>1.637</v>
+      </c>
+      <c r="O38" s="189">
         <f t="shared" si="4"/>
         <v>3.0862720439219007E-5</v>
       </c>
-      <c r="O38" s="196">
-        <f t="shared" ref="O38" si="24">AVERAGE(N38:N42)</f>
+      <c r="P38" s="196">
+        <f t="shared" ref="P38" si="42">AVERAGE(O38:O42)</f>
         <v>1.843359308412242E-5</v>
       </c>
-      <c r="P38" s="203">
-        <f t="shared" ref="P38" si="25">Q38/SQRT(5)</f>
+      <c r="Q38" s="279">
+        <f t="shared" ref="Q38" si="43">AVERAGE(M38:M42)</f>
+        <v>220.00505634962161</v>
+      </c>
+      <c r="R38" s="279">
+        <f t="shared" ref="R38" si="44">AVERAGE(N38:N42)</f>
+        <v>1.8046</v>
+      </c>
+      <c r="S38" s="279">
+        <f t="shared" ref="S38" si="45">SQRT(T38^2+((SQRT((0.5/D38)^2+(R38/Q38)^2+(0.06/225)^2))*P38)^2)</f>
+        <v>3.820488923827413E-6</v>
+      </c>
+      <c r="T38" s="203">
+        <f t="shared" ref="T38" si="46">U38/SQRT(5)</f>
         <v>3.8173859957856402E-6</v>
       </c>
-      <c r="Q38" s="199">
-        <f t="shared" ref="Q38" si="26">_xlfn.STDEV.S(N38:N42)</f>
+      <c r="U38" s="199">
+        <f t="shared" ref="U38" si="47">_xlfn.STDEV.S(O38:O42)</f>
         <v>8.5359345829324183E-6</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A39" s="116"/>
       <c r="B39" s="168">
         <v>2</v>
@@ -11778,7 +12134,7 @@
         <v>50</v>
       </c>
       <c r="D39" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>323.14999999999998</v>
       </c>
       <c r="E39" s="173">
@@ -11811,15 +12167,21 @@
         <f t="shared" si="3"/>
         <v>138.79668049792531</v>
       </c>
-      <c r="N39" s="183">
+      <c r="N39" s="238">
+        <v>1.589</v>
+      </c>
+      <c r="O39" s="183">
         <f t="shared" si="4"/>
         <v>1.1629376034248156E-5</v>
       </c>
-      <c r="O39" s="196"/>
-      <c r="P39" s="203"/>
-      <c r="Q39" s="199"/>
+      <c r="P39" s="196"/>
+      <c r="Q39" s="280"/>
+      <c r="R39" s="280"/>
+      <c r="S39" s="280"/>
+      <c r="T39" s="203"/>
+      <c r="U39" s="199"/>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A40" s="116"/>
       <c r="B40" s="168">
         <v>3</v>
@@ -11828,7 +12190,7 @@
         <v>50</v>
       </c>
       <c r="D40" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>323.14999999999998</v>
       </c>
       <c r="E40" s="173">
@@ -11861,15 +12223,21 @@
         <f t="shared" si="3"/>
         <v>142.60869565217391</v>
       </c>
-      <c r="N40" s="183">
+      <c r="N40" s="238">
+        <v>1.2370000000000001</v>
+      </c>
+      <c r="O40" s="183">
         <f t="shared" si="4"/>
         <v>1.1948773857870259E-5</v>
       </c>
-      <c r="O40" s="196"/>
-      <c r="P40" s="203"/>
-      <c r="Q40" s="199"/>
+      <c r="P40" s="196"/>
+      <c r="Q40" s="280"/>
+      <c r="R40" s="280"/>
+      <c r="S40" s="280"/>
+      <c r="T40" s="203"/>
+      <c r="U40" s="199"/>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A41" s="128"/>
       <c r="B41" s="171">
         <v>4</v>
@@ -11878,7 +12246,7 @@
         <v>50</v>
       </c>
       <c r="D41" s="53">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>323.14999999999998</v>
       </c>
       <c r="E41" s="173">
@@ -11911,15 +12279,21 @@
         <f t="shared" si="3"/>
         <v>283.75527426160335</v>
       </c>
-      <c r="N41" s="183">
+      <c r="N41" s="238">
+        <v>3.1930000000000001</v>
+      </c>
+      <c r="O41" s="183">
         <f t="shared" si="4"/>
         <v>2.3775041119508106E-5</v>
       </c>
-      <c r="O41" s="196"/>
-      <c r="P41" s="203"/>
-      <c r="Q41" s="199"/>
+      <c r="P41" s="196"/>
+      <c r="Q41" s="280"/>
+      <c r="R41" s="280"/>
+      <c r="S41" s="280"/>
+      <c r="T41" s="203"/>
+      <c r="U41" s="199"/>
     </row>
-    <row r="42" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="129"/>
       <c r="B42" s="170">
         <v>5</v>
@@ -11928,13 +12302,13 @@
         <v>50</v>
       </c>
       <c r="D42" s="54">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>323.14999999999998</v>
       </c>
       <c r="E42" s="174">
         <v>49.8</v>
       </c>
-      <c r="F42" s="274">
+      <c r="F42" s="277">
         <f t="shared" si="1"/>
         <v>322.95</v>
       </c>
@@ -11961,30 +12335,56 @@
         <f t="shared" si="3"/>
         <v>166.51785714285717</v>
       </c>
-      <c r="N42" s="185">
+      <c r="N42" s="239">
+        <v>1.367</v>
+      </c>
+      <c r="O42" s="185">
         <f t="shared" si="4"/>
         <v>1.3952053969766572E-5</v>
       </c>
-      <c r="O42" s="197"/>
-      <c r="P42" s="204"/>
-      <c r="Q42" s="200"/>
+      <c r="P42" s="197"/>
+      <c r="Q42" s="281"/>
+      <c r="R42" s="281"/>
+      <c r="S42" s="281"/>
+      <c r="T42" s="204"/>
+      <c r="U42" s="200"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="Q28:Q32"/>
-    <mergeCell ref="Q33:Q37"/>
+  <mergeCells count="57">
     <mergeCell ref="Q38:Q42"/>
-    <mergeCell ref="Q8:Q12"/>
     <mergeCell ref="Q13:Q17"/>
     <mergeCell ref="Q18:Q22"/>
     <mergeCell ref="Q23:Q27"/>
-    <mergeCell ref="O33:O37"/>
-    <mergeCell ref="O38:O42"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="Q28:Q32"/>
+    <mergeCell ref="Q33:Q37"/>
+    <mergeCell ref="S3:S7"/>
+    <mergeCell ref="S8:S12"/>
+    <mergeCell ref="S13:S17"/>
+    <mergeCell ref="S18:S22"/>
+    <mergeCell ref="S23:S27"/>
+    <mergeCell ref="S28:S32"/>
+    <mergeCell ref="S33:S37"/>
+    <mergeCell ref="S38:S42"/>
+    <mergeCell ref="R3:R7"/>
+    <mergeCell ref="R8:R12"/>
+    <mergeCell ref="R13:R17"/>
+    <mergeCell ref="R18:R22"/>
+    <mergeCell ref="R23:R27"/>
+    <mergeCell ref="U28:U32"/>
+    <mergeCell ref="U33:U37"/>
+    <mergeCell ref="U38:U42"/>
+    <mergeCell ref="U8:U12"/>
+    <mergeCell ref="U13:U17"/>
+    <mergeCell ref="U18:U22"/>
+    <mergeCell ref="U23:U27"/>
+    <mergeCell ref="P33:P37"/>
+    <mergeCell ref="P38:P42"/>
+    <mergeCell ref="A1:U1"/>
     <mergeCell ref="A3:A7"/>
-    <mergeCell ref="O3:O7"/>
+    <mergeCell ref="P3:P7"/>
+    <mergeCell ref="U3:U7"/>
+    <mergeCell ref="T3:T7"/>
     <mergeCell ref="Q3:Q7"/>
-    <mergeCell ref="P3:P7"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A13:A17"/>
     <mergeCell ref="A18:A22"/>
@@ -11992,23 +12392,27 @@
     <mergeCell ref="A38:A42"/>
     <mergeCell ref="A28:A32"/>
     <mergeCell ref="A33:A37"/>
-    <mergeCell ref="P33:P37"/>
-    <mergeCell ref="P38:P42"/>
-    <mergeCell ref="O8:O12"/>
-    <mergeCell ref="O13:O17"/>
-    <mergeCell ref="O18:O22"/>
-    <mergeCell ref="O23:O27"/>
-    <mergeCell ref="O28:O32"/>
+    <mergeCell ref="T33:T37"/>
+    <mergeCell ref="T38:T42"/>
     <mergeCell ref="P8:P12"/>
     <mergeCell ref="P13:P17"/>
     <mergeCell ref="P18:P22"/>
     <mergeCell ref="P23:P27"/>
     <mergeCell ref="P28:P32"/>
+    <mergeCell ref="T8:T12"/>
+    <mergeCell ref="T13:T17"/>
+    <mergeCell ref="T18:T22"/>
+    <mergeCell ref="T23:T27"/>
+    <mergeCell ref="T28:T32"/>
+    <mergeCell ref="R28:R32"/>
+    <mergeCell ref="R33:R37"/>
+    <mergeCell ref="R38:R42"/>
+    <mergeCell ref="Q8:Q12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <ignoredErrors>
-    <ignoredError sqref="O3:O42 Q3:Q42" formulaRange="1"/>
+    <ignoredError sqref="P3:P42 U3:U42" formulaRange="1"/>
   </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -12074,16 +12478,16 @@
       <c r="R1" s="138"/>
       <c r="S1" s="220"/>
       <c r="T1" s="175"/>
-      <c r="AG1" s="261" t="s">
+      <c r="AG1" s="264" t="s">
         <v>61</v>
       </c>
-      <c r="AH1" s="262"/>
-      <c r="AI1" s="262"/>
-      <c r="AJ1" s="262"/>
-      <c r="AK1" s="262"/>
-      <c r="AL1" s="262"/>
-      <c r="AM1" s="262"/>
-      <c r="AN1" s="263"/>
+      <c r="AH1" s="265"/>
+      <c r="AI1" s="265"/>
+      <c r="AJ1" s="265"/>
+      <c r="AK1" s="265"/>
+      <c r="AL1" s="265"/>
+      <c r="AM1" s="265"/>
+      <c r="AN1" s="266"/>
     </row>
     <row r="2" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="226" t="s">
@@ -12137,35 +12541,35 @@
       <c r="Q2" s="228" t="s">
         <v>57</v>
       </c>
-      <c r="R2" s="237" t="s">
+      <c r="R2" s="240" t="s">
         <v>58</v>
       </c>
-      <c r="S2" s="241" t="s">
+      <c r="S2" s="244" t="s">
         <v>59</v>
       </c>
       <c r="T2" s="99"/>
-      <c r="AG2" s="256" t="s">
+      <c r="AG2" s="259" t="s">
         <v>4</v>
       </c>
-      <c r="AH2" s="257" t="s">
+      <c r="AH2" s="260" t="s">
         <v>5</v>
       </c>
-      <c r="AI2" s="257" t="s">
+      <c r="AI2" s="260" t="s">
         <v>64</v>
       </c>
-      <c r="AJ2" s="258" t="s">
+      <c r="AJ2" s="261" t="s">
         <v>65</v>
       </c>
-      <c r="AK2" s="257" t="s">
+      <c r="AK2" s="260" t="s">
         <v>63</v>
       </c>
-      <c r="AL2" s="258" t="s">
+      <c r="AL2" s="261" t="s">
         <v>60</v>
       </c>
-      <c r="AM2" s="259" t="s">
+      <c r="AM2" s="262" t="s">
         <v>60</v>
       </c>
-      <c r="AN2" s="260" t="s">
+      <c r="AN2" s="263" t="s">
         <v>62</v>
       </c>
     </row>
@@ -12229,40 +12633,40 @@
         <f>_xlfn.STDEV.S(N3:N7)</f>
         <v>3.6872643964940771E-7</v>
       </c>
-      <c r="R3" s="238">
+      <c r="R3" s="241">
         <f>1/D3</f>
         <v>3.4704147145583901E-3</v>
       </c>
-      <c r="S3" s="242">
+      <c r="S3" s="245">
         <f>LN(O3)</f>
         <v>-13.180753833192105</v>
       </c>
-      <c r="AG3" s="247">
+      <c r="AG3" s="250">
         <v>1</v>
       </c>
-      <c r="AH3" s="248">
+      <c r="AH3" s="251">
         <v>1</v>
       </c>
-      <c r="AI3" s="270">
+      <c r="AI3" s="273">
         <f>Q3/SQRT(5)</f>
         <v>1.6489947683150986E-7</v>
       </c>
-      <c r="AJ3" s="270">
+      <c r="AJ3" s="273">
         <f>AI3/O3</f>
         <v>8.7407346233789304E-2</v>
       </c>
-      <c r="AK3" s="264">
+      <c r="AK3" s="267">
         <f>C3+273.15</f>
         <v>288.14999999999998</v>
       </c>
       <c r="AL3" s="235">
         <v>0.5</v>
       </c>
-      <c r="AM3" s="253">
+      <c r="AM3" s="256">
         <f>AVERAGE(AL3:AL7)</f>
         <v>0.52999999999999992</v>
       </c>
-      <c r="AN3" s="267">
+      <c r="AN3" s="270">
         <f>AM3/AK3^2</f>
         <v>6.3832024942423963E-6</v>
       </c>
@@ -12316,20 +12720,20 @@
       <c r="O4" s="215"/>
       <c r="P4" s="216"/>
       <c r="Q4" s="217"/>
-      <c r="R4" s="239"/>
-      <c r="S4" s="243"/>
-      <c r="AG4" s="249"/>
-      <c r="AH4" s="250">
+      <c r="R4" s="242"/>
+      <c r="S4" s="246"/>
+      <c r="AG4" s="252"/>
+      <c r="AH4" s="253">
         <v>2</v>
       </c>
-      <c r="AI4" s="265"/>
-      <c r="AJ4" s="271"/>
-      <c r="AK4" s="265"/>
+      <c r="AI4" s="268"/>
+      <c r="AJ4" s="274"/>
+      <c r="AK4" s="268"/>
       <c r="AL4" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM4" s="254"/>
-      <c r="AN4" s="268"/>
+      <c r="AM4" s="257"/>
+      <c r="AN4" s="271"/>
     </row>
     <row r="5" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="116"/>
@@ -12380,20 +12784,20 @@
       <c r="O5" s="215"/>
       <c r="P5" s="216"/>
       <c r="Q5" s="217"/>
-      <c r="R5" s="239"/>
-      <c r="S5" s="243"/>
-      <c r="AG5" s="249"/>
-      <c r="AH5" s="250">
+      <c r="R5" s="242"/>
+      <c r="S5" s="246"/>
+      <c r="AG5" s="252"/>
+      <c r="AH5" s="253">
         <v>3</v>
       </c>
-      <c r="AI5" s="265"/>
-      <c r="AJ5" s="271"/>
-      <c r="AK5" s="265"/>
+      <c r="AI5" s="268"/>
+      <c r="AJ5" s="274"/>
+      <c r="AK5" s="268"/>
       <c r="AL5" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM5" s="254"/>
-      <c r="AN5" s="268"/>
+      <c r="AM5" s="257"/>
+      <c r="AN5" s="271"/>
     </row>
     <row r="6" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="116"/>
@@ -12444,20 +12848,20 @@
       <c r="O6" s="215"/>
       <c r="P6" s="216"/>
       <c r="Q6" s="217"/>
-      <c r="R6" s="239"/>
-      <c r="S6" s="243"/>
-      <c r="AG6" s="249"/>
-      <c r="AH6" s="250">
+      <c r="R6" s="242"/>
+      <c r="S6" s="246"/>
+      <c r="AG6" s="252"/>
+      <c r="AH6" s="253">
         <v>4</v>
       </c>
-      <c r="AI6" s="265"/>
-      <c r="AJ6" s="271"/>
-      <c r="AK6" s="265"/>
+      <c r="AI6" s="268"/>
+      <c r="AJ6" s="274"/>
+      <c r="AK6" s="268"/>
       <c r="AL6" s="218">
         <v>0.64999999999999947</v>
       </c>
-      <c r="AM6" s="254"/>
-      <c r="AN6" s="268"/>
+      <c r="AM6" s="257"/>
+      <c r="AN6" s="271"/>
     </row>
     <row r="7" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="129"/>
@@ -12508,20 +12912,20 @@
       <c r="O7" s="222"/>
       <c r="P7" s="223"/>
       <c r="Q7" s="224"/>
-      <c r="R7" s="240"/>
-      <c r="S7" s="244"/>
-      <c r="AG7" s="251"/>
-      <c r="AH7" s="252">
+      <c r="R7" s="243"/>
+      <c r="S7" s="247"/>
+      <c r="AG7" s="254"/>
+      <c r="AH7" s="255">
         <v>5</v>
       </c>
-      <c r="AI7" s="266"/>
-      <c r="AJ7" s="272"/>
-      <c r="AK7" s="266"/>
+      <c r="AI7" s="269"/>
+      <c r="AJ7" s="275"/>
+      <c r="AK7" s="269"/>
       <c r="AL7" s="225">
         <v>0.5</v>
       </c>
-      <c r="AM7" s="255"/>
-      <c r="AN7" s="269"/>
+      <c r="AM7" s="258"/>
+      <c r="AN7" s="272"/>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A8" s="137">
@@ -12583,40 +12987,40 @@
         <f t="shared" ref="Q8" si="7">_xlfn.STDEV.S(N8:N12)</f>
         <v>9.882695021731592E-7</v>
       </c>
-      <c r="R8" s="238">
+      <c r="R8" s="241">
         <f t="shared" ref="R4:R42" si="8">1/D8</f>
         <v>3.4112229234180458E-3</v>
       </c>
-      <c r="S8" s="242">
+      <c r="S8" s="245">
         <f t="shared" ref="S8:S38" si="9">LN(O8)</f>
         <v>-13.181573232616515</v>
       </c>
-      <c r="AG8" s="247">
+      <c r="AG8" s="250">
         <v>2</v>
       </c>
-      <c r="AH8" s="248">
+      <c r="AH8" s="251">
         <v>1</v>
       </c>
-      <c r="AI8" s="270">
+      <c r="AI8" s="273">
         <f t="shared" ref="AI8:AI42" si="10">Q8/SQRT(5)</f>
         <v>4.4196755738981199E-7</v>
       </c>
-      <c r="AJ8" s="270">
+      <c r="AJ8" s="273">
         <f t="shared" ref="AJ8" si="11">AI8/O8</f>
         <v>0.23446331923193769</v>
       </c>
-      <c r="AK8" s="264">
+      <c r="AK8" s="267">
         <f>C8+273.15</f>
         <v>293.14999999999998</v>
       </c>
       <c r="AL8" s="235">
         <v>0.59999999999999964</v>
       </c>
-      <c r="AM8" s="253">
+      <c r="AM8" s="256">
         <f t="shared" ref="AM8" si="12">AVERAGE(AL8:AL12)</f>
         <v>0.66000000000000014</v>
       </c>
-      <c r="AN8" s="267">
+      <c r="AN8" s="270">
         <f t="shared" ref="AN8" si="13">AM8/AK8^2</f>
         <v>7.6800516099468215E-6</v>
       </c>
@@ -12670,20 +13074,20 @@
       <c r="O9" s="215"/>
       <c r="P9" s="216"/>
       <c r="Q9" s="217"/>
-      <c r="R9" s="239"/>
-      <c r="S9" s="243"/>
-      <c r="AG9" s="249"/>
-      <c r="AH9" s="250">
+      <c r="R9" s="242"/>
+      <c r="S9" s="246"/>
+      <c r="AG9" s="252"/>
+      <c r="AH9" s="253">
         <v>2</v>
       </c>
-      <c r="AI9" s="265"/>
-      <c r="AJ9" s="271"/>
-      <c r="AK9" s="265"/>
+      <c r="AI9" s="268"/>
+      <c r="AJ9" s="274"/>
+      <c r="AK9" s="268"/>
       <c r="AL9" s="218">
         <v>0.70000000000000107</v>
       </c>
-      <c r="AM9" s="254"/>
-      <c r="AN9" s="268"/>
+      <c r="AM9" s="257"/>
+      <c r="AN9" s="271"/>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A10" s="116"/>
@@ -12734,20 +13138,20 @@
       <c r="O10" s="215"/>
       <c r="P10" s="216"/>
       <c r="Q10" s="217"/>
-      <c r="R10" s="239"/>
-      <c r="S10" s="243"/>
-      <c r="AG10" s="249"/>
-      <c r="AH10" s="250">
+      <c r="R10" s="242"/>
+      <c r="S10" s="246"/>
+      <c r="AG10" s="252"/>
+      <c r="AH10" s="253">
         <v>3</v>
       </c>
-      <c r="AI10" s="265"/>
-      <c r="AJ10" s="271"/>
-      <c r="AK10" s="265"/>
+      <c r="AI10" s="268"/>
+      <c r="AJ10" s="274"/>
+      <c r="AK10" s="268"/>
       <c r="AL10" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM10" s="254"/>
-      <c r="AN10" s="268"/>
+      <c r="AM10" s="257"/>
+      <c r="AN10" s="271"/>
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A11" s="116"/>
@@ -12798,20 +13202,20 @@
       <c r="O11" s="215"/>
       <c r="P11" s="216"/>
       <c r="Q11" s="217"/>
-      <c r="R11" s="239"/>
-      <c r="S11" s="243"/>
-      <c r="AG11" s="249"/>
-      <c r="AH11" s="250">
+      <c r="R11" s="242"/>
+      <c r="S11" s="246"/>
+      <c r="AG11" s="252"/>
+      <c r="AH11" s="253">
         <v>4</v>
       </c>
-      <c r="AI11" s="265"/>
-      <c r="AJ11" s="271"/>
-      <c r="AK11" s="265"/>
+      <c r="AI11" s="268"/>
+      <c r="AJ11" s="274"/>
+      <c r="AK11" s="268"/>
       <c r="AL11" s="218">
         <v>1</v>
       </c>
-      <c r="AM11" s="254"/>
-      <c r="AN11" s="268"/>
+      <c r="AM11" s="257"/>
+      <c r="AN11" s="271"/>
     </row>
     <row r="12" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="129"/>
@@ -12862,20 +13266,20 @@
       <c r="O12" s="222"/>
       <c r="P12" s="223"/>
       <c r="Q12" s="224"/>
-      <c r="R12" s="240"/>
-      <c r="S12" s="244"/>
-      <c r="AG12" s="251"/>
-      <c r="AH12" s="252">
+      <c r="R12" s="243"/>
+      <c r="S12" s="247"/>
+      <c r="AG12" s="254"/>
+      <c r="AH12" s="255">
         <v>5</v>
       </c>
-      <c r="AI12" s="266"/>
-      <c r="AJ12" s="272"/>
-      <c r="AK12" s="266"/>
+      <c r="AI12" s="269"/>
+      <c r="AJ12" s="275"/>
+      <c r="AK12" s="269"/>
       <c r="AL12" s="225">
         <v>0.5</v>
       </c>
-      <c r="AM12" s="255"/>
-      <c r="AN12" s="269"/>
+      <c r="AM12" s="258"/>
+      <c r="AN12" s="272"/>
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A13" s="137">
@@ -12937,40 +13341,40 @@
         <f t="shared" ref="Q13" si="17">_xlfn.STDEV.S(N13:N17)</f>
         <v>6.3719058620950689E-7</v>
       </c>
-      <c r="R13" s="238">
+      <c r="R13" s="241">
         <f t="shared" si="8"/>
         <v>3.3540164346805303E-3</v>
       </c>
-      <c r="S13" s="242">
+      <c r="S13" s="245">
         <f t="shared" si="9"/>
         <v>-12.594567433546684</v>
       </c>
-      <c r="AG13" s="247">
+      <c r="AG13" s="250">
         <v>3</v>
       </c>
-      <c r="AH13" s="248">
+      <c r="AH13" s="251">
         <v>1</v>
       </c>
-      <c r="AI13" s="270">
+      <c r="AI13" s="273">
         <f t="shared" ref="AI13:AI42" si="18">Q13/SQRT(5)</f>
         <v>2.8496029307747946E-7</v>
       </c>
-      <c r="AJ13" s="270">
+      <c r="AJ13" s="273">
         <f t="shared" ref="AJ13" si="19">AI13/O13</f>
         <v>8.4049568299715591E-2</v>
       </c>
-      <c r="AK13" s="264">
+      <c r="AK13" s="267">
         <f>C13+273.15</f>
         <v>298.14999999999998</v>
       </c>
       <c r="AL13" s="235">
         <v>0.5</v>
       </c>
-      <c r="AM13" s="253">
+      <c r="AM13" s="256">
         <f t="shared" ref="AM13" si="20">AVERAGE(AL13:AL17)</f>
         <v>0.51000000000000012</v>
       </c>
-      <c r="AN13" s="267">
+      <c r="AN13" s="270">
         <f t="shared" ref="AN13" si="21">AM13/AK13^2</f>
         <v>5.7372073844946202E-6</v>
       </c>
@@ -13024,20 +13428,20 @@
       <c r="O14" s="215"/>
       <c r="P14" s="216"/>
       <c r="Q14" s="217"/>
-      <c r="R14" s="239"/>
-      <c r="S14" s="243"/>
-      <c r="AG14" s="249"/>
-      <c r="AH14" s="250">
+      <c r="R14" s="242"/>
+      <c r="S14" s="246"/>
+      <c r="AG14" s="252"/>
+      <c r="AH14" s="253">
         <v>2</v>
       </c>
-      <c r="AI14" s="265"/>
-      <c r="AJ14" s="271"/>
-      <c r="AK14" s="265"/>
+      <c r="AI14" s="268"/>
+      <c r="AJ14" s="274"/>
+      <c r="AK14" s="268"/>
       <c r="AL14" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM14" s="254"/>
-      <c r="AN14" s="268"/>
+      <c r="AM14" s="257"/>
+      <c r="AN14" s="271"/>
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A15" s="116"/>
@@ -13088,20 +13492,20 @@
       <c r="O15" s="215"/>
       <c r="P15" s="216"/>
       <c r="Q15" s="217"/>
-      <c r="R15" s="239"/>
-      <c r="S15" s="243"/>
-      <c r="AG15" s="249"/>
-      <c r="AH15" s="250">
+      <c r="R15" s="242"/>
+      <c r="S15" s="246"/>
+      <c r="AG15" s="252"/>
+      <c r="AH15" s="253">
         <v>3</v>
       </c>
-      <c r="AI15" s="265"/>
-      <c r="AJ15" s="271"/>
-      <c r="AK15" s="265"/>
+      <c r="AI15" s="268"/>
+      <c r="AJ15" s="274"/>
+      <c r="AK15" s="268"/>
       <c r="AL15" s="218">
         <v>0.55000000000000071</v>
       </c>
-      <c r="AM15" s="254"/>
-      <c r="AN15" s="268"/>
+      <c r="AM15" s="257"/>
+      <c r="AN15" s="271"/>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A16" s="116"/>
@@ -13152,20 +13556,20 @@
       <c r="O16" s="215"/>
       <c r="P16" s="216"/>
       <c r="Q16" s="217"/>
-      <c r="R16" s="239"/>
-      <c r="S16" s="243"/>
-      <c r="AG16" s="249"/>
-      <c r="AH16" s="250">
+      <c r="R16" s="242"/>
+      <c r="S16" s="246"/>
+      <c r="AG16" s="252"/>
+      <c r="AH16" s="253">
         <v>4</v>
       </c>
-      <c r="AI16" s="265"/>
-      <c r="AJ16" s="271"/>
-      <c r="AK16" s="265"/>
+      <c r="AI16" s="268"/>
+      <c r="AJ16" s="274"/>
+      <c r="AK16" s="268"/>
       <c r="AL16" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM16" s="254"/>
-      <c r="AN16" s="268"/>
+      <c r="AM16" s="257"/>
+      <c r="AN16" s="271"/>
     </row>
     <row r="17" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="129"/>
@@ -13216,20 +13620,20 @@
       <c r="O17" s="222"/>
       <c r="P17" s="223"/>
       <c r="Q17" s="224"/>
-      <c r="R17" s="240"/>
-      <c r="S17" s="244"/>
-      <c r="AG17" s="251"/>
-      <c r="AH17" s="252">
+      <c r="R17" s="243"/>
+      <c r="S17" s="247"/>
+      <c r="AG17" s="254"/>
+      <c r="AH17" s="255">
         <v>5</v>
       </c>
-      <c r="AI17" s="266"/>
-      <c r="AJ17" s="272"/>
-      <c r="AK17" s="266"/>
+      <c r="AI17" s="269"/>
+      <c r="AJ17" s="275"/>
+      <c r="AK17" s="269"/>
       <c r="AL17" s="225">
         <v>0.5</v>
       </c>
-      <c r="AM17" s="255"/>
-      <c r="AN17" s="269"/>
+      <c r="AM17" s="258"/>
+      <c r="AN17" s="272"/>
     </row>
     <row r="18" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A18" s="137">
@@ -13291,40 +13695,40 @@
         <f t="shared" ref="Q18" si="24">_xlfn.STDEV.S(N18:N22)</f>
         <v>2.6673929684094582E-6</v>
       </c>
-      <c r="R18" s="238">
+      <c r="R18" s="241">
         <f t="shared" si="8"/>
         <v>3.298697014679202E-3</v>
       </c>
-      <c r="S18" s="242">
+      <c r="S18" s="245">
         <f t="shared" si="9"/>
         <v>-11.794917543679352</v>
       </c>
-      <c r="AG18" s="247">
+      <c r="AG18" s="250">
         <v>4</v>
       </c>
-      <c r="AH18" s="248">
+      <c r="AH18" s="251">
         <v>1</v>
       </c>
-      <c r="AI18" s="270">
+      <c r="AI18" s="273">
         <f t="shared" ref="AI18:AI42" si="25">Q18/SQRT(5)</f>
         <v>1.1928944000136995E-6</v>
       </c>
-      <c r="AJ18" s="270">
+      <c r="AJ18" s="273">
         <f t="shared" ref="AJ18" si="26">AI18/O18</f>
         <v>0.15815014831466895</v>
       </c>
-      <c r="AK18" s="264">
+      <c r="AK18" s="267">
         <f>C18+273.15</f>
         <v>303.14999999999998</v>
       </c>
       <c r="AL18" s="235">
         <v>0.5</v>
       </c>
-      <c r="AM18" s="253">
+      <c r="AM18" s="256">
         <f t="shared" ref="AM18" si="27">AVERAGE(AL18:AL22)</f>
         <v>0.50999999999999979</v>
       </c>
-      <c r="AN18" s="267">
+      <c r="AN18" s="270">
         <f t="shared" ref="AN18" si="28">AM18/AK18^2</f>
         <v>5.549515017273272E-6</v>
       </c>
@@ -13378,20 +13782,20 @@
       <c r="O19" s="215"/>
       <c r="P19" s="216"/>
       <c r="Q19" s="217"/>
-      <c r="R19" s="239"/>
-      <c r="S19" s="243"/>
-      <c r="AG19" s="249"/>
-      <c r="AH19" s="250">
+      <c r="R19" s="242"/>
+      <c r="S19" s="246"/>
+      <c r="AG19" s="252"/>
+      <c r="AH19" s="253">
         <v>2</v>
       </c>
-      <c r="AI19" s="265"/>
-      <c r="AJ19" s="271"/>
-      <c r="AK19" s="265"/>
+      <c r="AI19" s="268"/>
+      <c r="AJ19" s="274"/>
+      <c r="AK19" s="268"/>
       <c r="AL19" s="218">
         <v>0.54999999999999893</v>
       </c>
-      <c r="AM19" s="254"/>
-      <c r="AN19" s="268"/>
+      <c r="AM19" s="257"/>
+      <c r="AN19" s="271"/>
     </row>
     <row r="20" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A20" s="116"/>
@@ -13442,20 +13846,20 @@
       <c r="O20" s="215"/>
       <c r="P20" s="216"/>
       <c r="Q20" s="217"/>
-      <c r="R20" s="239"/>
-      <c r="S20" s="243"/>
-      <c r="AG20" s="249"/>
-      <c r="AH20" s="250">
+      <c r="R20" s="242"/>
+      <c r="S20" s="246"/>
+      <c r="AG20" s="252"/>
+      <c r="AH20" s="253">
         <v>3</v>
       </c>
-      <c r="AI20" s="265"/>
-      <c r="AJ20" s="271"/>
-      <c r="AK20" s="265"/>
+      <c r="AI20" s="268"/>
+      <c r="AJ20" s="274"/>
+      <c r="AK20" s="268"/>
       <c r="AL20" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM20" s="254"/>
-      <c r="AN20" s="268"/>
+      <c r="AM20" s="257"/>
+      <c r="AN20" s="271"/>
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A21" s="116"/>
@@ -13506,20 +13910,20 @@
       <c r="O21" s="215"/>
       <c r="P21" s="216"/>
       <c r="Q21" s="217"/>
-      <c r="R21" s="239"/>
-      <c r="S21" s="243"/>
-      <c r="AG21" s="249"/>
-      <c r="AH21" s="250">
+      <c r="R21" s="242"/>
+      <c r="S21" s="246"/>
+      <c r="AG21" s="252"/>
+      <c r="AH21" s="253">
         <v>4</v>
       </c>
-      <c r="AI21" s="265"/>
-      <c r="AJ21" s="271"/>
-      <c r="AK21" s="265"/>
+      <c r="AI21" s="268"/>
+      <c r="AJ21" s="274"/>
+      <c r="AK21" s="268"/>
       <c r="AL21" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM21" s="254"/>
-      <c r="AN21" s="268"/>
+      <c r="AM21" s="257"/>
+      <c r="AN21" s="271"/>
     </row>
     <row r="22" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="129"/>
@@ -13570,20 +13974,20 @@
       <c r="O22" s="222"/>
       <c r="P22" s="223"/>
       <c r="Q22" s="224"/>
-      <c r="R22" s="240"/>
-      <c r="S22" s="244"/>
-      <c r="AG22" s="251"/>
-      <c r="AH22" s="252">
+      <c r="R22" s="243"/>
+      <c r="S22" s="247"/>
+      <c r="AG22" s="254"/>
+      <c r="AH22" s="255">
         <v>5</v>
       </c>
-      <c r="AI22" s="266"/>
-      <c r="AJ22" s="272"/>
-      <c r="AK22" s="266"/>
+      <c r="AI22" s="269"/>
+      <c r="AJ22" s="275"/>
+      <c r="AK22" s="269"/>
       <c r="AL22" s="225">
         <v>0.5</v>
       </c>
-      <c r="AM22" s="255"/>
-      <c r="AN22" s="269"/>
+      <c r="AM22" s="258"/>
+      <c r="AN22" s="272"/>
     </row>
     <row r="23" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A23" s="137">
@@ -13645,40 +14049,40 @@
         <f t="shared" ref="Q23" si="31">_xlfn.STDEV.S(N23:N27)</f>
         <v>2.0709701812871915E-6</v>
       </c>
-      <c r="R23" s="238">
+      <c r="R23" s="241">
         <f t="shared" si="8"/>
         <v>3.2451728054518907E-3</v>
       </c>
-      <c r="S23" s="242">
+      <c r="S23" s="245">
         <f t="shared" si="9"/>
         <v>-11.664435498815054</v>
       </c>
-      <c r="AG23" s="247">
+      <c r="AG23" s="250">
         <v>5</v>
       </c>
-      <c r="AH23" s="248">
+      <c r="AH23" s="251">
         <v>1</v>
       </c>
-      <c r="AI23" s="270">
+      <c r="AI23" s="273">
         <f t="shared" ref="AI23:AI42" si="32">Q23/SQRT(5)</f>
         <v>9.2616602094664455E-7</v>
       </c>
-      <c r="AJ23" s="270">
+      <c r="AJ23" s="273">
         <f t="shared" ref="AJ23" si="33">AI23/O23</f>
         <v>0.10776774990414704</v>
       </c>
-      <c r="AK23" s="264">
+      <c r="AK23" s="267">
         <f>C23+273.15</f>
         <v>308.14999999999998</v>
       </c>
       <c r="AL23" s="235">
         <v>0.5</v>
       </c>
-      <c r="AM23" s="253">
+      <c r="AM23" s="256">
         <f t="shared" ref="AM23" si="34">AVERAGE(AL23:AL27)</f>
         <v>0.60000000000000075</v>
       </c>
-      <c r="AN23" s="267">
+      <c r="AN23" s="270">
         <f t="shared" ref="AN23" si="35">AM23/AK23^2</f>
         <v>6.3186879223467043E-6</v>
       </c>
@@ -13732,20 +14136,20 @@
       <c r="O24" s="215"/>
       <c r="P24" s="216"/>
       <c r="Q24" s="217"/>
-      <c r="R24" s="239"/>
-      <c r="S24" s="243"/>
-      <c r="AG24" s="249"/>
-      <c r="AH24" s="250">
+      <c r="R24" s="242"/>
+      <c r="S24" s="246"/>
+      <c r="AG24" s="252"/>
+      <c r="AH24" s="253">
         <v>2</v>
       </c>
-      <c r="AI24" s="265"/>
-      <c r="AJ24" s="271"/>
-      <c r="AK24" s="265"/>
+      <c r="AI24" s="268"/>
+      <c r="AJ24" s="274"/>
+      <c r="AK24" s="268"/>
       <c r="AL24" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM24" s="254"/>
-      <c r="AN24" s="268"/>
+      <c r="AM24" s="257"/>
+      <c r="AN24" s="271"/>
     </row>
     <row r="25" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A25" s="116"/>
@@ -13796,20 +14200,20 @@
       <c r="O25" s="215"/>
       <c r="P25" s="216"/>
       <c r="Q25" s="217"/>
-      <c r="R25" s="239"/>
-      <c r="S25" s="243"/>
-      <c r="AG25" s="249"/>
-      <c r="AH25" s="250">
+      <c r="R25" s="242"/>
+      <c r="S25" s="246"/>
+      <c r="AG25" s="252"/>
+      <c r="AH25" s="253">
         <v>3</v>
       </c>
-      <c r="AI25" s="265"/>
-      <c r="AJ25" s="271"/>
-      <c r="AK25" s="265"/>
+      <c r="AI25" s="268"/>
+      <c r="AJ25" s="274"/>
+      <c r="AK25" s="268"/>
       <c r="AL25" s="218">
         <v>0.90000000000000213</v>
       </c>
-      <c r="AM25" s="254"/>
-      <c r="AN25" s="268"/>
+      <c r="AM25" s="257"/>
+      <c r="AN25" s="271"/>
     </row>
     <row r="26" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A26" s="116"/>
@@ -13860,20 +14264,20 @@
       <c r="O26" s="215"/>
       <c r="P26" s="216"/>
       <c r="Q26" s="217"/>
-      <c r="R26" s="239"/>
-      <c r="S26" s="243"/>
-      <c r="AG26" s="249"/>
-      <c r="AH26" s="250">
+      <c r="R26" s="242"/>
+      <c r="S26" s="246"/>
+      <c r="AG26" s="252"/>
+      <c r="AH26" s="253">
         <v>4</v>
       </c>
-      <c r="AI26" s="265"/>
-      <c r="AJ26" s="271"/>
-      <c r="AK26" s="265"/>
+      <c r="AI26" s="268"/>
+      <c r="AJ26" s="274"/>
+      <c r="AK26" s="268"/>
       <c r="AL26" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM26" s="254"/>
-      <c r="AN26" s="268"/>
+      <c r="AM26" s="257"/>
+      <c r="AN26" s="271"/>
     </row>
     <row r="27" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="129"/>
@@ -13924,20 +14328,20 @@
       <c r="O27" s="222"/>
       <c r="P27" s="223"/>
       <c r="Q27" s="224"/>
-      <c r="R27" s="240"/>
-      <c r="S27" s="244"/>
-      <c r="AG27" s="251"/>
-      <c r="AH27" s="252">
+      <c r="R27" s="243"/>
+      <c r="S27" s="247"/>
+      <c r="AG27" s="254"/>
+      <c r="AH27" s="255">
         <v>5</v>
       </c>
-      <c r="AI27" s="266"/>
-      <c r="AJ27" s="272"/>
-      <c r="AK27" s="266"/>
+      <c r="AI27" s="269"/>
+      <c r="AJ27" s="275"/>
+      <c r="AK27" s="269"/>
       <c r="AL27" s="225">
         <v>0.60000000000000142</v>
       </c>
-      <c r="AM27" s="255"/>
-      <c r="AN27" s="269"/>
+      <c r="AM27" s="258"/>
+      <c r="AN27" s="272"/>
     </row>
     <row r="28" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A28" s="137">
@@ -13999,40 +14403,40 @@
         <f t="shared" ref="Q28" si="38">_xlfn.STDEV.S(N28:N32)</f>
         <v>2.7014714463734948E-6</v>
       </c>
-      <c r="R28" s="238">
+      <c r="R28" s="241">
         <f t="shared" si="8"/>
         <v>3.1933578157432542E-3</v>
       </c>
-      <c r="S28" s="242">
+      <c r="S28" s="245">
         <f t="shared" si="9"/>
         <v>-11.631005742844986</v>
       </c>
-      <c r="AG28" s="247">
+      <c r="AG28" s="250">
         <v>6</v>
       </c>
-      <c r="AH28" s="248">
+      <c r="AH28" s="251">
         <v>1</v>
       </c>
-      <c r="AI28" s="270">
+      <c r="AI28" s="273">
         <f t="shared" ref="AI28:AI42" si="39">Q28/SQRT(5)</f>
         <v>1.2081347586731623E-6</v>
       </c>
-      <c r="AJ28" s="270">
+      <c r="AJ28" s="273">
         <f t="shared" ref="AJ28" si="40">AI28/O28</f>
         <v>0.13595556607935072</v>
       </c>
-      <c r="AK28" s="264">
+      <c r="AK28" s="267">
         <f>C28+273.15</f>
         <v>313.14999999999998</v>
       </c>
       <c r="AL28" s="235">
         <v>0.55000000000000071</v>
       </c>
-      <c r="AM28" s="253">
+      <c r="AM28" s="256">
         <f t="shared" ref="AM28" si="41">AVERAGE(AL28:AL32)</f>
         <v>0.74000000000000055</v>
       </c>
-      <c r="AN28" s="267">
+      <c r="AN28" s="270">
         <f t="shared" ref="AN28" si="42">AM28/AK28^2</f>
         <v>7.5461752631327161E-6</v>
       </c>
@@ -14086,20 +14490,20 @@
       <c r="O29" s="215"/>
       <c r="P29" s="216"/>
       <c r="Q29" s="217"/>
-      <c r="R29" s="239"/>
-      <c r="S29" s="243"/>
-      <c r="AG29" s="249"/>
-      <c r="AH29" s="250">
+      <c r="R29" s="242"/>
+      <c r="S29" s="246"/>
+      <c r="AG29" s="252"/>
+      <c r="AH29" s="253">
         <v>2</v>
       </c>
-      <c r="AI29" s="265"/>
-      <c r="AJ29" s="271"/>
-      <c r="AK29" s="265"/>
+      <c r="AI29" s="268"/>
+      <c r="AJ29" s="274"/>
+      <c r="AK29" s="268"/>
       <c r="AL29" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM29" s="254"/>
-      <c r="AN29" s="268"/>
+      <c r="AM29" s="257"/>
+      <c r="AN29" s="271"/>
     </row>
     <row r="30" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A30" s="116"/>
@@ -14150,20 +14554,20 @@
       <c r="O30" s="215"/>
       <c r="P30" s="216"/>
       <c r="Q30" s="217"/>
-      <c r="R30" s="239"/>
-      <c r="S30" s="243"/>
-      <c r="AG30" s="249"/>
-      <c r="AH30" s="250">
+      <c r="R30" s="242"/>
+      <c r="S30" s="246"/>
+      <c r="AG30" s="252"/>
+      <c r="AH30" s="253">
         <v>3</v>
       </c>
-      <c r="AI30" s="265"/>
-      <c r="AJ30" s="271"/>
-      <c r="AK30" s="265"/>
+      <c r="AI30" s="268"/>
+      <c r="AJ30" s="274"/>
+      <c r="AK30" s="268"/>
       <c r="AL30" s="218">
         <v>1.6000000000000014</v>
       </c>
-      <c r="AM30" s="254"/>
-      <c r="AN30" s="268"/>
+      <c r="AM30" s="257"/>
+      <c r="AN30" s="271"/>
     </row>
     <row r="31" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A31" s="116"/>
@@ -14214,20 +14618,20 @@
       <c r="O31" s="215"/>
       <c r="P31" s="216"/>
       <c r="Q31" s="217"/>
-      <c r="R31" s="239"/>
-      <c r="S31" s="243"/>
-      <c r="AG31" s="249"/>
-      <c r="AH31" s="250">
+      <c r="R31" s="242"/>
+      <c r="S31" s="246"/>
+      <c r="AG31" s="252"/>
+      <c r="AH31" s="253">
         <v>4</v>
       </c>
-      <c r="AI31" s="265"/>
-      <c r="AJ31" s="271"/>
-      <c r="AK31" s="265"/>
+      <c r="AI31" s="268"/>
+      <c r="AJ31" s="274"/>
+      <c r="AK31" s="268"/>
       <c r="AL31" s="218">
         <v>0.55000000000000071</v>
       </c>
-      <c r="AM31" s="254"/>
-      <c r="AN31" s="268"/>
+      <c r="AM31" s="257"/>
+      <c r="AN31" s="271"/>
     </row>
     <row r="32" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="129"/>
@@ -14278,20 +14682,20 @@
       <c r="O32" s="222"/>
       <c r="P32" s="223"/>
       <c r="Q32" s="224"/>
-      <c r="R32" s="240"/>
-      <c r="S32" s="244"/>
-      <c r="AG32" s="251"/>
-      <c r="AH32" s="252">
+      <c r="R32" s="243"/>
+      <c r="S32" s="247"/>
+      <c r="AG32" s="254"/>
+      <c r="AH32" s="255">
         <v>5</v>
       </c>
-      <c r="AI32" s="266"/>
-      <c r="AJ32" s="272"/>
-      <c r="AK32" s="266"/>
+      <c r="AI32" s="269"/>
+      <c r="AJ32" s="275"/>
+      <c r="AK32" s="269"/>
       <c r="AL32" s="225">
         <v>0.5</v>
       </c>
-      <c r="AM32" s="255"/>
-      <c r="AN32" s="269"/>
+      <c r="AM32" s="258"/>
+      <c r="AN32" s="272"/>
     </row>
     <row r="33" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A33" s="137">
@@ -14353,40 +14757,40 @@
         <f t="shared" ref="Q33" si="45">_xlfn.STDEV.S(N33:N37)</f>
         <v>6.0580013453342243E-6</v>
       </c>
-      <c r="R33" s="238">
+      <c r="R33" s="241">
         <f t="shared" si="8"/>
         <v>3.1431714600031434E-3</v>
       </c>
-      <c r="S33" s="242">
+      <c r="S33" s="245">
         <f t="shared" si="9"/>
         <v>-11.257812904279829</v>
       </c>
-      <c r="AG33" s="247">
+      <c r="AG33" s="250">
         <v>7</v>
       </c>
-      <c r="AH33" s="248">
+      <c r="AH33" s="251">
         <v>1</v>
       </c>
-      <c r="AI33" s="270">
+      <c r="AI33" s="273">
         <f t="shared" ref="AI33:AI42" si="46">Q33/SQRT(5)</f>
         <v>2.7092205631905007E-6</v>
       </c>
-      <c r="AJ33" s="270">
+      <c r="AJ33" s="273">
         <f t="shared" ref="AJ33" si="47">AI33/O33</f>
         <v>0.20991834121988498</v>
       </c>
-      <c r="AK33" s="264">
+      <c r="AK33" s="267">
         <f>C33+273.15</f>
         <v>318.14999999999998</v>
       </c>
       <c r="AL33" s="235">
         <v>0.5</v>
       </c>
-      <c r="AM33" s="253">
+      <c r="AM33" s="256">
         <f t="shared" ref="AM33" si="48">AVERAGE(AL33:AL37)</f>
         <v>0.55000000000000004</v>
       </c>
-      <c r="AN33" s="267">
+      <c r="AN33" s="270">
         <f t="shared" ref="AN33" si="49">AM33/AK33^2</f>
         <v>5.4337397548380613E-6</v>
       </c>
@@ -14440,20 +14844,20 @@
       <c r="O34" s="215"/>
       <c r="P34" s="216"/>
       <c r="Q34" s="217"/>
-      <c r="R34" s="239"/>
-      <c r="S34" s="243"/>
-      <c r="AG34" s="249"/>
-      <c r="AH34" s="250">
+      <c r="R34" s="242"/>
+      <c r="S34" s="246"/>
+      <c r="AG34" s="252"/>
+      <c r="AH34" s="253">
         <v>2</v>
       </c>
-      <c r="AI34" s="265"/>
-      <c r="AJ34" s="271"/>
-      <c r="AK34" s="265"/>
+      <c r="AI34" s="268"/>
+      <c r="AJ34" s="274"/>
+      <c r="AK34" s="268"/>
       <c r="AL34" s="218">
         <v>0.64999999999999858</v>
       </c>
-      <c r="AM34" s="254"/>
-      <c r="AN34" s="268"/>
+      <c r="AM34" s="257"/>
+      <c r="AN34" s="271"/>
     </row>
     <row r="35" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A35" s="116"/>
@@ -14504,20 +14908,20 @@
       <c r="O35" s="215"/>
       <c r="P35" s="216"/>
       <c r="Q35" s="217"/>
-      <c r="R35" s="239"/>
-      <c r="S35" s="243"/>
-      <c r="AG35" s="249"/>
-      <c r="AH35" s="250">
+      <c r="R35" s="242"/>
+      <c r="S35" s="246"/>
+      <c r="AG35" s="252"/>
+      <c r="AH35" s="253">
         <v>3</v>
       </c>
-      <c r="AI35" s="265"/>
-      <c r="AJ35" s="271"/>
-      <c r="AK35" s="265"/>
+      <c r="AI35" s="268"/>
+      <c r="AJ35" s="274"/>
+      <c r="AK35" s="268"/>
       <c r="AL35" s="218">
         <v>0.55000000000000071</v>
       </c>
-      <c r="AM35" s="254"/>
-      <c r="AN35" s="268"/>
+      <c r="AM35" s="257"/>
+      <c r="AN35" s="271"/>
     </row>
     <row r="36" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A36" s="116"/>
@@ -14568,20 +14972,20 @@
       <c r="O36" s="215"/>
       <c r="P36" s="216"/>
       <c r="Q36" s="217"/>
-      <c r="R36" s="239"/>
-      <c r="S36" s="243"/>
-      <c r="AG36" s="249"/>
-      <c r="AH36" s="250">
+      <c r="R36" s="242"/>
+      <c r="S36" s="246"/>
+      <c r="AG36" s="252"/>
+      <c r="AH36" s="253">
         <v>4</v>
       </c>
-      <c r="AI36" s="265"/>
-      <c r="AJ36" s="271"/>
-      <c r="AK36" s="265"/>
+      <c r="AI36" s="268"/>
+      <c r="AJ36" s="274"/>
+      <c r="AK36" s="268"/>
       <c r="AL36" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM36" s="254"/>
-      <c r="AN36" s="268"/>
+      <c r="AM36" s="257"/>
+      <c r="AN36" s="271"/>
     </row>
     <row r="37" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="129"/>
@@ -14632,20 +15036,20 @@
       <c r="O37" s="222"/>
       <c r="P37" s="223"/>
       <c r="Q37" s="224"/>
-      <c r="R37" s="240"/>
-      <c r="S37" s="244"/>
-      <c r="AG37" s="251"/>
-      <c r="AH37" s="252">
+      <c r="R37" s="243"/>
+      <c r="S37" s="247"/>
+      <c r="AG37" s="254"/>
+      <c r="AH37" s="255">
         <v>5</v>
       </c>
-      <c r="AI37" s="266"/>
-      <c r="AJ37" s="272"/>
-      <c r="AK37" s="266"/>
+      <c r="AI37" s="269"/>
+      <c r="AJ37" s="275"/>
+      <c r="AK37" s="269"/>
       <c r="AL37" s="225">
         <v>0.55000000000000071</v>
       </c>
-      <c r="AM37" s="255"/>
-      <c r="AN37" s="269"/>
+      <c r="AM37" s="258"/>
+      <c r="AN37" s="272"/>
     </row>
     <row r="38" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A38" s="137">
@@ -14707,40 +15111,40 @@
         <f t="shared" ref="Q38" si="52">_xlfn.STDEV.S(N38:N42)</f>
         <v>8.5359345829324183E-6</v>
       </c>
-      <c r="R38" s="238">
+      <c r="R38" s="241">
         <f t="shared" si="8"/>
         <v>3.0945381401825778E-3</v>
       </c>
-      <c r="S38" s="242">
+      <c r="S38" s="245">
         <f t="shared" si="9"/>
         <v>-10.901335846840498</v>
       </c>
-      <c r="AG38" s="247">
+      <c r="AG38" s="250">
         <v>8</v>
       </c>
-      <c r="AH38" s="248">
+      <c r="AH38" s="251">
         <v>1</v>
       </c>
-      <c r="AI38" s="270">
+      <c r="AI38" s="273">
         <f t="shared" ref="AI38:AI42" si="53">Q38/SQRT(5)</f>
         <v>3.8173859957856402E-6</v>
       </c>
-      <c r="AJ38" s="270">
+      <c r="AJ38" s="273">
         <f t="shared" ref="AJ38" si="54">AI38/O38</f>
         <v>0.20708854634931184</v>
       </c>
-      <c r="AK38" s="264">
+      <c r="AK38" s="267">
         <f>C38+273.15</f>
         <v>323.14999999999998</v>
       </c>
       <c r="AL38" s="235">
         <v>0.5</v>
       </c>
-      <c r="AM38" s="253">
+      <c r="AM38" s="256">
         <f t="shared" ref="AM38" si="55">AVERAGE(AL38:AL42)</f>
         <v>0.5</v>
       </c>
-      <c r="AN38" s="267">
+      <c r="AN38" s="270">
         <f t="shared" ref="AN38" si="56">AM38/AK38^2</f>
         <v>4.7880831505223246E-6</v>
       </c>
@@ -14794,20 +15198,20 @@
       <c r="O39" s="215"/>
       <c r="P39" s="216"/>
       <c r="Q39" s="217"/>
-      <c r="R39" s="239"/>
-      <c r="S39" s="243"/>
-      <c r="AG39" s="249"/>
-      <c r="AH39" s="250">
+      <c r="R39" s="242"/>
+      <c r="S39" s="246"/>
+      <c r="AG39" s="252"/>
+      <c r="AH39" s="253">
         <v>2</v>
       </c>
-      <c r="AI39" s="265"/>
-      <c r="AJ39" s="271"/>
-      <c r="AK39" s="265"/>
+      <c r="AI39" s="268"/>
+      <c r="AJ39" s="274"/>
+      <c r="AK39" s="268"/>
       <c r="AL39" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM39" s="254"/>
-      <c r="AN39" s="268"/>
+      <c r="AM39" s="257"/>
+      <c r="AN39" s="271"/>
     </row>
     <row r="40" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A40" s="116"/>
@@ -14858,20 +15262,20 @@
       <c r="O40" s="215"/>
       <c r="P40" s="216"/>
       <c r="Q40" s="217"/>
-      <c r="R40" s="239"/>
-      <c r="S40" s="243"/>
-      <c r="AG40" s="249"/>
-      <c r="AH40" s="250">
+      <c r="R40" s="242"/>
+      <c r="S40" s="246"/>
+      <c r="AG40" s="252"/>
+      <c r="AH40" s="253">
         <v>3</v>
       </c>
-      <c r="AI40" s="265"/>
-      <c r="AJ40" s="271"/>
-      <c r="AK40" s="265"/>
+      <c r="AI40" s="268"/>
+      <c r="AJ40" s="274"/>
+      <c r="AK40" s="268"/>
       <c r="AL40" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM40" s="254"/>
-      <c r="AN40" s="268"/>
+      <c r="AM40" s="257"/>
+      <c r="AN40" s="271"/>
     </row>
     <row r="41" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A41" s="116"/>
@@ -14922,20 +15326,20 @@
       <c r="O41" s="215"/>
       <c r="P41" s="216"/>
       <c r="Q41" s="217"/>
-      <c r="R41" s="239"/>
-      <c r="S41" s="243"/>
-      <c r="AG41" s="249"/>
-      <c r="AH41" s="250">
+      <c r="R41" s="242"/>
+      <c r="S41" s="246"/>
+      <c r="AG41" s="252"/>
+      <c r="AH41" s="253">
         <v>4</v>
       </c>
-      <c r="AI41" s="265"/>
-      <c r="AJ41" s="271"/>
-      <c r="AK41" s="265"/>
+      <c r="AI41" s="268"/>
+      <c r="AJ41" s="274"/>
+      <c r="AK41" s="268"/>
       <c r="AL41" s="218">
         <v>0.5</v>
       </c>
-      <c r="AM41" s="254"/>
-      <c r="AN41" s="268"/>
+      <c r="AM41" s="257"/>
+      <c r="AN41" s="271"/>
     </row>
     <row r="42" spans="1:40" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="129"/>
@@ -14986,20 +15390,20 @@
       <c r="O42" s="222"/>
       <c r="P42" s="223"/>
       <c r="Q42" s="224"/>
-      <c r="R42" s="240"/>
-      <c r="S42" s="244"/>
-      <c r="AG42" s="251"/>
-      <c r="AH42" s="252">
+      <c r="R42" s="243"/>
+      <c r="S42" s="247"/>
+      <c r="AG42" s="254"/>
+      <c r="AH42" s="255">
         <v>5</v>
       </c>
-      <c r="AI42" s="266"/>
-      <c r="AJ42" s="272"/>
-      <c r="AK42" s="266"/>
+      <c r="AI42" s="269"/>
+      <c r="AJ42" s="275"/>
+      <c r="AK42" s="269"/>
       <c r="AL42" s="225">
         <v>0.5</v>
       </c>
-      <c r="AM42" s="255"/>
-      <c r="AN42" s="269"/>
+      <c r="AM42" s="258"/>
+      <c r="AN42" s="272"/>
     </row>
     <row r="44" spans="1:40" x14ac:dyDescent="0.2">
       <c r="G44" s="115"/>
@@ -15120,17 +15524,17 @@
   <dimension ref="A1:C113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="275"/>
+    <col min="1" max="16384" width="10.83203125" style="278"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="275" t="s">
+      <c r="A1" s="278" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="275" t="s">
+      <c r="B1" s="278" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="278" t="s">
         <v>49</v>
       </c>
     </row>
@@ -90804,206 +91208,206 @@
       <c r="A308" s="114" t="s">
         <v>60</v>
       </c>
-      <c r="B308" s="245">
+      <c r="B308" s="248">
         <f>MAX(0.5, ((MAX(B5:B305))-(MIN(B5:B305)))/2)</f>
         <v>0.5</v>
       </c>
-      <c r="C308" s="245"/>
-      <c r="D308" s="245">
+      <c r="C308" s="248"/>
+      <c r="D308" s="248">
         <f t="shared" ref="C308:BN308" si="0">MAX(0.5, ((MAX(D5:D305))-(MIN(D5:D305)))/2)</f>
         <v>0.5</v>
       </c>
-      <c r="E308" s="245"/>
-      <c r="F308" s="245">
+      <c r="E308" s="248"/>
+      <c r="F308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="G308" s="245"/>
-      <c r="H308" s="245">
+      <c r="G308" s="248"/>
+      <c r="H308" s="248">
         <f t="shared" si="0"/>
         <v>0.64999999999999947</v>
       </c>
-      <c r="I308" s="245"/>
-      <c r="J308" s="245">
+      <c r="I308" s="248"/>
+      <c r="J308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="K308" s="245"/>
-      <c r="L308" s="245">
+      <c r="K308" s="248"/>
+      <c r="L308" s="248">
         <f t="shared" si="0"/>
         <v>0.59999999999999964</v>
       </c>
-      <c r="M308" s="245"/>
-      <c r="N308" s="245">
+      <c r="M308" s="248"/>
+      <c r="N308" s="248">
         <f t="shared" si="0"/>
         <v>0.70000000000000107</v>
       </c>
-      <c r="O308" s="245"/>
-      <c r="P308" s="245">
+      <c r="O308" s="248"/>
+      <c r="P308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="Q308" s="245"/>
-      <c r="R308" s="245">
+      <c r="Q308" s="248"/>
+      <c r="R308" s="248">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="S308" s="245"/>
-      <c r="T308" s="245">
+      <c r="S308" s="248"/>
+      <c r="T308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="U308" s="245"/>
-      <c r="V308" s="245">
+      <c r="U308" s="248"/>
+      <c r="V308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="W308" s="245"/>
-      <c r="X308" s="245">
+      <c r="W308" s="248"/>
+      <c r="X308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="Y308" s="245"/>
-      <c r="Z308" s="245">
+      <c r="Y308" s="248"/>
+      <c r="Z308" s="248">
         <f t="shared" si="0"/>
         <v>0.55000000000000071</v>
       </c>
-      <c r="AA308" s="245"/>
-      <c r="AB308" s="245">
+      <c r="AA308" s="248"/>
+      <c r="AB308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AC308" s="245"/>
-      <c r="AD308" s="245">
+      <c r="AC308" s="248"/>
+      <c r="AD308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AE308" s="245"/>
-      <c r="AF308" s="245">
+      <c r="AE308" s="248"/>
+      <c r="AF308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AG308" s="245"/>
-      <c r="AH308" s="245">
+      <c r="AG308" s="248"/>
+      <c r="AH308" s="248">
         <f t="shared" si="0"/>
         <v>0.54999999999999893</v>
       </c>
-      <c r="AI308" s="245"/>
-      <c r="AJ308" s="245">
+      <c r="AI308" s="248"/>
+      <c r="AJ308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AK308" s="245"/>
-      <c r="AL308" s="245">
+      <c r="AK308" s="248"/>
+      <c r="AL308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AM308" s="245"/>
-      <c r="AN308" s="245">
+      <c r="AM308" s="248"/>
+      <c r="AN308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AO308" s="245"/>
-      <c r="AP308" s="245">
+      <c r="AO308" s="248"/>
+      <c r="AP308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AQ308" s="245"/>
-      <c r="AR308" s="245">
+      <c r="AQ308" s="248"/>
+      <c r="AR308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AS308" s="245"/>
-      <c r="AT308" s="245">
+      <c r="AS308" s="248"/>
+      <c r="AT308" s="248">
         <f t="shared" si="0"/>
         <v>0.90000000000000213</v>
       </c>
-      <c r="AU308" s="245"/>
-      <c r="AV308" s="245">
+      <c r="AU308" s="248"/>
+      <c r="AV308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="AW308" s="245"/>
-      <c r="AX308" s="245">
+      <c r="AW308" s="248"/>
+      <c r="AX308" s="248">
         <f t="shared" si="0"/>
         <v>0.60000000000000142</v>
       </c>
-      <c r="AY308" s="245"/>
-      <c r="AZ308" s="245">
+      <c r="AY308" s="248"/>
+      <c r="AZ308" s="248">
         <f t="shared" si="0"/>
         <v>0.55000000000000071</v>
       </c>
-      <c r="BA308" s="245"/>
-      <c r="BB308" s="245">
+      <c r="BA308" s="248"/>
+      <c r="BB308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="BC308" s="245"/>
-      <c r="BD308" s="245">
+      <c r="BC308" s="248"/>
+      <c r="BD308" s="248">
         <f t="shared" si="0"/>
         <v>1.6000000000000014</v>
       </c>
-      <c r="BE308" s="245"/>
-      <c r="BF308" s="245">
+      <c r="BE308" s="248"/>
+      <c r="BF308" s="248">
         <f t="shared" si="0"/>
         <v>0.55000000000000071</v>
       </c>
-      <c r="BG308" s="245"/>
-      <c r="BH308" s="245">
+      <c r="BG308" s="248"/>
+      <c r="BH308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="BI308" s="245"/>
-      <c r="BJ308" s="245">
+      <c r="BI308" s="248"/>
+      <c r="BJ308" s="248">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="BK308" s="245"/>
-      <c r="BL308" s="245">
+      <c r="BK308" s="248"/>
+      <c r="BL308" s="248">
         <f t="shared" si="0"/>
         <v>0.64999999999999858</v>
       </c>
-      <c r="BM308" s="245"/>
-      <c r="BN308" s="245">
+      <c r="BM308" s="248"/>
+      <c r="BN308" s="248">
         <f t="shared" si="0"/>
         <v>0.55000000000000071</v>
       </c>
-      <c r="BO308" s="245"/>
-      <c r="BP308" s="245">
+      <c r="BO308" s="248"/>
+      <c r="BP308" s="248">
         <f t="shared" ref="BO308:CC308" si="1">MAX(0.5, ((MAX(BP5:BP305))-(MIN(BP5:BP305)))/2)</f>
         <v>0.5</v>
       </c>
-      <c r="BQ308" s="245"/>
-      <c r="BR308" s="245">
+      <c r="BQ308" s="248"/>
+      <c r="BR308" s="248">
         <f t="shared" si="1"/>
         <v>0.55000000000000071</v>
       </c>
-      <c r="BS308" s="245"/>
-      <c r="BT308" s="245">
+      <c r="BS308" s="248"/>
+      <c r="BT308" s="248">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="BU308" s="245"/>
-      <c r="BV308" s="245">
+      <c r="BU308" s="248"/>
+      <c r="BV308" s="248">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="BW308" s="245"/>
-      <c r="BX308" s="245">
+      <c r="BW308" s="248"/>
+      <c r="BX308" s="248">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="BY308" s="245"/>
-      <c r="BZ308" s="245">
+      <c r="BY308" s="248"/>
+      <c r="BZ308" s="248">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="CA308" s="245"/>
-      <c r="CB308" s="245">
+      <c r="CA308" s="248"/>
+      <c r="CB308" s="248">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="CC308" s="246"/>
+      <c r="CC308" s="249"/>
     </row>
   </sheetData>
   <mergeCells count="50">

</xml_diff>